<commit_message>
docs: prepare ClaimTrace final submission
</commit_message>
<xml_diff>
--- a/evaluation/manual_review_20.xlsx
+++ b/evaluation/manual_review_20.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核记录" sheetId="1" r:id="R49fbf3044a514011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R6e7b13f7bbac4d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核记录" sheetId="1" r:id="R539c21922ea6490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R5e54bd72fab342da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -596,16 +596,7 @@
     <x:t xml:space="preserve">test_full.csv没有保存next_action，因此20条均只能如实标记为无法核查，不能补造建议。</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">确认方式</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">逐行阅读J至Q列。同意时把P列改为“已确认”；不同意时修改N、Q列并把P列设为“需修改”。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">当前状态</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CLAIM031已确认；其余19条为根据现有结果和官方页面预填的待审建议，不能冒充本人已完成人工复核。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">禁止修改</x:t>
@@ -789,7 +780,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -832,6 +823,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1120,6 +1120,13 @@
     <x:col min="17" max="17" width="72" customWidth="1"/>
     <x:col min="18" max="18" width="42" customWidth="1"/>
     <x:col min="19" max="19" width="48" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="26" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="20" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18.75">
@@ -1147,7 +1154,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>10条案例改写 + 10条合成新文案。20条均已完成人工复核确认；复核结论不等于法律批准，正式发布仍需人工确认。</x:v>
+        <x:v>10条案例改写 + 10条合成新文案。20条均已完成人工复核和结构化编码；复核结论不等于法律批准，正式发布仍需人工确认。</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1219,14 +1226,14 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J4" s="5" t="n">
-        <x:f>COUNTIF(P7:P26,"已确认")</x:f>
+        <x:f>COUNTIF(Z7:Z26,"completed")</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="K4" s="5" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="L4" s="6" t="n">
-        <x:f>COUNTIF(P7:P26,"待确认")</x:f>
+        <x:f>COUNTIF(Z7:Z26,"pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M4" s="2"/>
@@ -1316,6 +1323,27 @@
       <x:c r="S6" s="7" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="T6" s="19" t="str">
+        <x:v>citation_present</x:v>
+      </x:c>
+      <x:c r="U6" s="19" t="str">
+        <x:v>citation_supported</x:v>
+      </x:c>
+      <x:c r="V6" s="19" t="str">
+        <x:v>reason_supported</x:v>
+      </x:c>
+      <x:c r="W6" s="19" t="str">
+        <x:v>recommendation_actionable</x:v>
+      </x:c>
+      <x:c r="X6" s="19" t="str">
+        <x:v>uncertainty_clear</x:v>
+      </x:c>
+      <x:c r="Y6" s="19" t="str">
+        <x:v>human_final_label</x:v>
+      </x:c>
+      <x:c r="Z6" s="19" t="str">
+        <x:v>review_status</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="9">
@@ -1375,6 +1403,27 @@
       <x:c r="S7" s="8" t="s">
         <x:v>40</x:v>
       </x:c>
+      <x:c r="T7" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U7" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V7" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="W7" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X7" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y7" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z7" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="9">
@@ -1434,6 +1483,27 @@
       <x:c r="S8" s="8" t="s">
         <x:v>40</x:v>
       </x:c>
+      <x:c r="T8" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U8" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V8" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W8" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X8" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y8" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z8" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="78" customHeight="1">
       <x:c r="A9" s="9">
@@ -1493,6 +1563,27 @@
       <x:c r="S9" s="8" t="s">
         <x:v>56</x:v>
       </x:c>
+      <x:c r="T9" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U9" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="V9" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="W9" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X9" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="Y9" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z9" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="78" customHeight="1">
       <x:c r="A10" s="9">
@@ -1552,6 +1643,27 @@
       <x:c r="S10" s="8" t="s">
         <x:v>66</x:v>
       </x:c>
+      <x:c r="T10" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U10" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V10" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="W10" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X10" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="Y10" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z10" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="78" customHeight="1">
       <x:c r="A11" s="9">
@@ -1611,6 +1723,27 @@
       <x:c r="S11" s="8" t="s">
         <x:v>75</x:v>
       </x:c>
+      <x:c r="T11" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U11" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V11" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W11" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X11" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y11" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z11" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="78" customHeight="1">
       <x:c r="A12" s="9">
@@ -1670,6 +1803,27 @@
       <x:c r="S12" s="8" t="s">
         <x:v>56</x:v>
       </x:c>
+      <x:c r="T12" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U12" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V12" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="W12" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X12" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="Y12" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z12" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="78" customHeight="1">
       <x:c r="A13" s="9">
@@ -1729,6 +1883,27 @@
       <x:c r="S13" s="8" t="s">
         <x:v>75</x:v>
       </x:c>
+      <x:c r="T13" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U13" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V13" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="W13" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X13" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="Y13" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z13" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="78" customHeight="1">
       <x:c r="A14" s="9">
@@ -1784,6 +1959,27 @@
       </x:c>
       <x:c r="R14" s="8"/>
       <x:c r="S14" s="8"/>
+      <x:c r="T14" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U14" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V14" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W14" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X14" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y14" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z14" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="78" customHeight="1">
       <x:c r="A15" s="9">
@@ -1843,6 +2039,27 @@
       <x:c r="S15" s="8" t="s">
         <x:v>111</x:v>
       </x:c>
+      <x:c r="T15" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U15" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V15" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W15" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X15" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y15" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z15" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="78" customHeight="1">
       <x:c r="A16" s="9">
@@ -1902,6 +2119,27 @@
       <x:c r="S16" s="8" t="s">
         <x:v>111</x:v>
       </x:c>
+      <x:c r="T16" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U16" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V16" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W16" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X16" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y16" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z16" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="78" customHeight="1">
       <x:c r="A17" s="9">
@@ -1957,6 +2195,27 @@
       </x:c>
       <x:c r="R17" s="8"/>
       <x:c r="S17" s="8"/>
+      <x:c r="T17" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U17" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V17" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W17" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X17" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y17" s="21" t="str">
+        <x:v>low_risk</x:v>
+      </x:c>
+      <x:c r="Z17" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="78" customHeight="1">
       <x:c r="A18" s="9">
@@ -2012,6 +2271,27 @@
       </x:c>
       <x:c r="R18" s="8"/>
       <x:c r="S18" s="8"/>
+      <x:c r="T18" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U18" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V18" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W18" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X18" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y18" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z18" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="78" customHeight="1">
       <x:c r="A19" s="9">
@@ -2071,6 +2351,27 @@
       <x:c r="S19" s="8" t="s">
         <x:v>141</x:v>
       </x:c>
+      <x:c r="T19" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U19" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V19" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W19" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X19" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y19" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z19" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="78" customHeight="1">
       <x:c r="A20" s="9">
@@ -2126,6 +2427,27 @@
       </x:c>
       <x:c r="R20" s="8"/>
       <x:c r="S20" s="8"/>
+      <x:c r="T20" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U20" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V20" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W20" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X20" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y20" s="21" t="str">
+        <x:v>low_risk</x:v>
+      </x:c>
+      <x:c r="Z20" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="78" customHeight="1">
       <x:c r="A21" s="9">
@@ -2181,6 +2503,27 @@
       </x:c>
       <x:c r="R21" s="8"/>
       <x:c r="S21" s="8"/>
+      <x:c r="T21" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U21" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V21" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W21" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X21" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y21" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z21" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="78" customHeight="1">
       <x:c r="A22" s="9">
@@ -2240,6 +2583,27 @@
       <x:c r="S22" s="8" t="s">
         <x:v>56</x:v>
       </x:c>
+      <x:c r="T22" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="U22" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="V22" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W22" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X22" s="21" t="str">
+        <x:v>uncertain</x:v>
+      </x:c>
+      <x:c r="Y22" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z22" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="78" customHeight="1">
       <x:c r="A23" s="9">
@@ -2295,6 +2659,27 @@
       </x:c>
       <x:c r="R23" s="8"/>
       <x:c r="S23" s="8"/>
+      <x:c r="T23" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U23" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V23" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="W23" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X23" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y23" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z23" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="78" customHeight="1">
       <x:c r="A24" s="9">
@@ -2350,6 +2735,27 @@
       </x:c>
       <x:c r="R24" s="8"/>
       <x:c r="S24" s="8"/>
+      <x:c r="T24" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U24" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V24" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W24" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X24" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y24" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z24" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="78" customHeight="1">
       <x:c r="A25" s="9">
@@ -2405,6 +2811,27 @@
       </x:c>
       <x:c r="R25" s="8"/>
       <x:c r="S25" s="8"/>
+      <x:c r="T25" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U25" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V25" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="W25" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X25" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y25" s="21" t="str">
+        <x:v>evidence_needed</x:v>
+      </x:c>
+      <x:c r="Z25" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="78" customHeight="1">
       <x:c r="A26" s="9">
@@ -2460,6 +2887,27 @@
       </x:c>
       <x:c r="R26" s="8"/>
       <x:c r="S26" s="8"/>
+      <x:c r="T26" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="U26" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="V26" s="21" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="W26" s="21" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="X26" s="21" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Y26" s="21" t="str">
+        <x:v>high_risk</x:v>
+      </x:c>
+      <x:c r="Z26" s="21" t="str">
+        <x:v>completed</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="P7:P26">
@@ -2467,14 +2915,32 @@
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="待确认"/>
     <x:cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="需修改"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="P7:P26">
       <x:formula1>"待确认,已确认,需修改"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="T7:T26">
+      <x:formula1>"yes,no,uncertain"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="U7:V26">
+      <x:formula1>"yes,no,uncertain,not_applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="W7:W26">
+      <x:formula1>"yes,no,uncertain,not_applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="X7:X26">
+      <x:formula1>"yes,no,uncertain,not_applicable"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Y7:Y26">
+      <x:formula1>"high_risk,evidence_needed,low_risk"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Z7:Z26">
+      <x:formula1>"completed,pending,needs_revision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e32d08e88bc4e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e20956d4a224274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2541,35 +3007,35 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="16" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="B8" s="13" t="s">
-        <x:v>196</x:v>
+      <x:c r="A8" s="16" t="str">
+        <x:v>结构化字段</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="str">
+        <x:v>复核记录T至Z列保存结构化结果。citation_supported、reason_supported和uncertainty_clear基于已确认的人工复核结论；无引用记录的citation_supported记为not_applicable。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="16" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="B9" s="13" t="s">
-        <x:v>198</x:v>
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>20条记录均已完成人工复核和结构化编码，review_status均为completed。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="16" t="s">
-        <x:v>199</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B10" s="13" t="s">
-        <x:v>200</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="17" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B11" s="14" t="s">
-        <x:v>202</x:v>
+        <x:v>199</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Prepare English presentation and final project documentation
Add English case summaries and a default English interface, refresh report
and screenshots, document verification, and remove obsolete review files.
</commit_message>
<xml_diff>
--- a/evaluation/manual_review_20.xlsx
+++ b/evaluation/manual_review_20.xlsx
@@ -905,9 +905,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ClaimTrace">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="ClaimTrace">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -957,7 +957,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="ClaimTrace">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>

<commit_message>
docs: translate review materials and evaluation scripts to English; keep report PDF only
</commit_message>
<xml_diff>
--- a/evaluation/manual_review_20.xlsx
+++ b/evaluation/manual_review_20.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核记录" sheetId="1" r:id="R539c21922ea6490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R5e54bd72fab342da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Review" sheetId="1" r:id="R8a3635ce28c14305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Notes" sheetId="2" r:id="R6b2d16431aae44a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11,90 +11,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t xml:space="preserve">ClaimTrace 锁定测试集人工复核（20条）</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">总样本</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">案例改写</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">合成新文案</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">系统转人工</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已确认</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">待确认</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">序号</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">claim_id</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">中文文案</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">样本类型</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">参考标签</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">系统输出</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">转人工</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">相似度</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">模型理由</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断支持</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">引用支持</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">建议可执行性</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不确定性表达</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">建议人工标签</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">系统评价</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">复核状态</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">复核说明</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">引用标题</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">引用链接</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM031</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">每月只花9元，这张流量卡就能不限量使用全部高速流量。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">case_derived</x:t>
   </x:si>
   <x:si>
@@ -104,511 +23,127 @@
     <x:t xml:space="preserve">high_risk</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">否</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim about unlimited high-speed data for only 9 yuan per month is similar to a previous case where a company made a false price claim regarding a mobile data card. This indicates a risk of misleading advertising.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">部分支持：低价且不限量属于需核验的量价承诺；相似案例只能提示风险，不能证明当前承诺虚假。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分支持：官方案例证明另一家公司“超大流量9元/月”与实际不符，只能支持同类风险，不能证明本卡不实。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无法核查：test_full.csv未保存next_action字段。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由使用风险措辞，但系统仍直接输出high_risk，未充分区分类比风险与当前事实。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">过度升级：参考标签要求证据，系统直接判高风险</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：部分支持：低价且不限量属于需核验的量价承诺；相似案例只能提示风险，不能证明当前承诺虚假。；引用：部分支持：官方案例证明另一家公司“超大流量9元/月”与实际不符，只能支持同类风险，不能证明本卡不实。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由使用风险措辞，但系统仍直接输出high_risk，未充分区分类比风险与当前事实。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">北京市昌平区市场监管局查处中智无线（北京）科技有限公司发布违法广告案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2025/art_1212b0d62d0844d58c635269e40efe35.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM032</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">使用这套护肤品七天，就能完全消除红肿、瘙痒和痘痘。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that the skincare product can completely eliminate symptoms such as redness, itching, and acne, which is a strong treatment promise. This is similar to a case where a cosmetic was advertised as treating skin conditions, leading to consumer confusion with pharmaceuticals.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：七天“完全消除”多种皮肤症状属于明确、绝对化的治疗效果承诺。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">直接相关：官方案例即化妆品宣称治疗红、肿、痒、刺痛和痘痘，与当前症状和产品类型高度一致。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由说明了相似案例和药品混淆风险，但未明确提示最终发布仍需人工结合产品事实确认。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">判断一致，引用直接相关</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：七天“完全消除”多种皮肤症状属于明确、绝对化的治疗效果承诺。；引用：直接相关：官方案例即化妆品宣称治疗红、肿、痒、刺痛和痘痘，与当前症状和产品类型高度一致。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由说明了相似案例和药品混淆风险，但未明确提示最终发布仍需人工结合产品事实确认。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">浙江省杭州市拱墅区市场监管局查处杭州迅犹贸易有限公司违法广告案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM034</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">已有大量消费者亲自证明，这款果冻可以快速减肥。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests a strong cure promise for weight loss, which is a high-risk assertion without sufficient evidence to support it. Similar cases have involved unsupported health claims that were deemed illegal.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">部分支持：快速减肥和“消费者证明”需要效果证据及评价真实性证明，尚不能仅凭文案认定虚假。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不足：理由将缺少证据直接推向高风险，没有充分说明仍需核验当前评价和产品效果。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">汕尾市城区某商贸行互联网食品广告案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.shanwei.gov.cn/swscjdglj/zwgk/0800/dxal/content/post_1074414.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM035</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">实测证明，这款家用美容仪能够显著提升皮肤紧致度。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests a significant improvement in skin firmness, which is a strong therapeutic promise that is likely to be considered a medical claim. This type of claim is often scrutinized and can be classified as a high risk due to potential consumer deception.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">部分支持：显著提升紧致度属于可验证的功效宣称，应有检测或试验依据；仅凭输入不能直接认定高风险。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">弱相关：来源案例是普通洗手液虚假宣称美白，能说明化妆品功效需真实依据，但与美容仪紧致功效并非同一产品或效果。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不足：理由把紧致功效概括成治疗性承诺，未说明产品属性和证据缺口。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">过度升级且引用较弱</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：部分支持：显著提升紧致度属于可验证的功效宣称，应有检测或试验依据；仅凭输入不能直接认定高风险。；引用：弱相关：来源案例是普通洗手液虚假宣称美白，能说明化妆品功效需真实依据，但与美容仪紧致功效并非同一产品或效果。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：不足：理由把紧致功效概括成治疗性承诺，未说明产品属性和证据缺口。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">房县某电子商务有限公司发布虚假化妆品广告案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/ggjgs/sjdt/gzdt/art/2024/art_93bcd60c81fb4145b6698014ba162cbb.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM036</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款普通膏体可以修复身体损伤并缓解相关疾病症状。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that the ordinary ointment can repair bodily injuries and alleviate disease symptoms, which is a medical claim for a non-medical product. This aligns with previous enforcement cases where similar claims were made for ordinary products, leading to legal action.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：普通膏体声称修复身体损伤、缓解疾病症状，属于明显的疾病治疗功能表达。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">直接相关：官方案例是普通膏体演绎疾病治疗和恢复活动能力，与当前普通膏体治疗性承诺高度一致。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由解释了普通产品使用医疗表述的风险，但仍应保留最终人工确认边界。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：普通膏体声称修复身体损伤、缓解疾病症状，属于明显的疾病治疗功能表达。；引用：直接相关：官方案例是普通膏体演绎疾病治疗和恢复活动能力，与当前普通膏体治疗性承诺高度一致。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由解释了普通产品使用医疗表述的风险，但仍应保留最终人工确认边界。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">山东省青岛市市场监管局查处青岛科曼奇商贸有限公司发布非医疗、药品、医疗器械广告使用医药用语行为案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2025/art_aa3fc21f7586462593b51175ba385186.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM037</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款产品可以全面改善身体机能，效果远超同类商品。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests comprehensive improvement of bodily functions, which is a strong health claim that is unsupported by evidence. Similar cases have been found where products made similar claims without scientific backing, leading to enforcement actions.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">部分支持：全面改善身体机能和远超同类的比较性功效需要证据，现有输入不足以直接认定高风险。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分相关：来源是普通食品虚假保健或改善功效案例，可支持需要证据，但与泛化的“全面改善身体机能”不完全相同。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不足：理由称缺少科学依据，却没有说明应先要求产品和比较证据。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">过度升级：更适合要求证据</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：部分支持：全面改善身体机能和远超同类的比较性功效需要证据，现有输入不足以直接认定高风险。；引用：部分相关：来源是普通食品虚假保健或改善功效案例，可支持需要证据，但与泛化的“全面改善身体机能”不完全相同。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：不足：理由称缺少科学依据，却没有说明应先要求产品和比较证据。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM039</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">本店销售的珍珠全部为天然珍珠，并附有真实权威证书。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim states that all pearls sold are natural and come with authentic certification. However, there is evidence of a case where fake pearls were sold as real, along with forged certification. This raises significant concerns about the authenticity of the pearls being sold.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">部分支持：天然珍珠和权威证书属于商品真实性承诺，需要当前店铺的鉴定与证书核验。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">高度相关但非直接证明：官方案例确有仿珍珠冒充真珍珠并伪造证书；只能提示核验，不能证明本店也造假。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不足：理由由旧案例推到当前商品真实性担忧，未充分强调不能跨商家直接证明。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">过度升级：类比风险不等于当前事实</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：部分支持：天然珍珠和权威证书属于商品真实性承诺，需要当前店铺的鉴定与证书核验。；引用：高度相关但非直接证明：官方案例确有仿珍珠冒充真珍珠并伪造证书；只能提示核验，不能证明本店也造假。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：不足：理由由旧案例推到当前商品真实性担忧，未充分强调不能跨商家直接证明。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">浙江省诸暨市市场监管局查处阮某某直播销售以假充真珍珠案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM040</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">直播间里的和田玉全部来自主播展示的矿区，来源绝对可靠。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">insufficient_evidence</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">是</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The retrieved evidence is below the provisional similarity threshold.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持转人工：矿区来源及“绝对可靠”需要供应链和产地凭证，检索分数低时转人工合理。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：相似度0.2928低于0.30暂定阈值，系统未提供来源，引用真实性无法核查。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统明确因低于暂定阈值转人工；但未提示人工应核验的产地和供应链材料。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">转人工合理</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持转人工：矿区来源及“绝对可靠”需要供应链和产地凭证，检索分数低时转人工合理。；引用：无引用：相似度0.2928低于0.30暂定阈值，系统未提供来源，引用真实性无法核查。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统明确因低于暂定阈值转人工；但未提示人工应核验的产地和供应链材料。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM042</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">权威研究和真实用户反馈证明，蜂王浆具有抗肿瘤等药理作用。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that royal jelly has anti-tumor properties, which is a medical claim that is prohibited for ordinary products. Similar cases have shown that such claims can lead to enforcement actions due to their misleading nature.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：普通蜂产品宣称抗肿瘤药理作用，属于明显的疾病治疗或药理功效表达。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">直接相关：官方案例明确指出蜂王浆“药理作用”、用户反馈、研究机构等内容不真实或违法，与输入高度一致。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由指出普通产品医疗宣称风险，但仍需人工核对具体产品属性和宣传语境。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：普通蜂产品宣称抗肿瘤药理作用，属于明显的疾病治疗或药理功效表达。；引用：直接相关：官方案例明确指出蜂王浆“药理作用”、用户反馈、研究机构等内容不真实或违法，与输入高度一致。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由指出普通产品医疗宣称风险，但仍需人工核对具体产品属性和宣传语境。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">杭州千岛湖春鑫蜂业有限公司广告违法案件</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2024/art_a68c3d6b97c24ec89fbb52182b9a24b8.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM044</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">每天饮用这款骆驼奶粉，就能有效控制血糖和三高问题。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that the product can control blood sugar and manage health issues related to 'three highs', which is a disease prevention or treatment claim. This is similar to a previous enforcement case where camel milk was advertised with similar health benefits, leading to legal action for making unapproved health claims.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：普通食品声称控制血糖和三高，属于疾病预防治疗功能表达。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">直接相关：官方案例明确涉及骆驼奶粉“降血糖”“调理三高”，与输入几乎同类。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由说明疾病治疗风险，但最终发布判断仍需人工确认产品属性和完整语境。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：普通食品声称控制血糖和三高，属于疾病预防治疗功能表达。；引用：直接相关：官方案例明确涉及骆驼奶粉“降血糖”“调理三高”，与输入几乎同类。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由说明疾病治疗风险，但最终发布判断仍需人工确认产品属性和完整语境。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">云南兴浩商贸有限公司广告违法案件</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM076</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款笔记本可选横线页或空白页。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">synthetic</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">low_risk</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；低风险判断仅基于输入内容，不等于法律批准。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统说明低于阈值并转人工，但没有区分普通商品规格信息。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM077</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款蓝牙音箱全年累计销量突破100万台。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">支持转人工：全年销量突破100万台是可核验事实，需要平台、订单或销售记录。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；销量真实性需另行查证。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统没有在证据不足时强行判断，但没有提示需要哪些销量凭证。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持转人工：全年销量突破100万台是可核验事实，需要平台、订单或销售记录。；引用：无引用：系统因低于阈值转人工，未生成来源；销量真实性需另行查证。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统没有在证据不足时强行判断，但没有提示需要哪些销量凭证。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM078</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款普通乳饮料可以治疗贫血。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that a regular dairy drink can treat a medical condition (anemia), which is a strong cure promise and is prohibited. Similar cases have established that such claims are illegal.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：普通乳饮料声称治疗贫血，是明确的疾病治疗承诺。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分相关：引用案例涉及普通食品宣称调节三高等疾病功能，支持普通食品不得宣称治疗疾病的风险；并非贫血或乳饮料同案。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由说明普通食品治疗疾病的风险，但“类似案例证明违法”的表述容易被理解为对当前商品的确定结论。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">判断一致，引用提供类别层面支持</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：普通乳饮料声称治疗贫血，是明确的疾病治疗承诺。；引用：部分相关：引用案例涉及普通食品宣称调节三高等疾病功能，支持普通食品不得宣称治疗疾病的风险；并非贫血或乳饮料同案。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由说明普通食品治疗疾病的风险，但“类似案例证明违法”的表述容易被理解为对当前商品的确定结论。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">海南恒昇医疗管理有限公司澄迈恒昇医院违法广告案</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2024/art_040ee3ac2e924c1e9735c6f47fb734d9.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM079</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款雨伞有黄色和黑色两种颜色。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim simply states the available colors of the umbrella, which does not raise any configured concerns or legal issues. This is not legal approval, but the claim appears to be straightforward and factual.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：仅描述雨伞颜色选项，未触发已配置风险；仍需确保商品页面与实物一致。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：低风险输出未附来源；颜色描述可直接核验，但低风险不等于法律批准。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">较清楚：模型说明不触发配置风险且不是法律批准。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">判断一致，无引用可以接受</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：仅描述雨伞颜色选项，未触发已配置风险；仍需确保商品页面与实物一致。；引用：无引用：低风险输出未附来源；颜色描述可直接核验，但低风险不等于法律批准。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：较清楚：模型说明不触发配置风险且不是法律批准。；人工结论：当前证据更支持low_risk。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM080</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这件防晒衣的防紫外线系数达到UPF50+。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">支持转人工：UPF50+是可验证的产品性能指标，需要检测报告、执行标准和适用条件。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；性能真实性需检测材料支持。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统说明低于阈值并转人工，但没有指出应核验测试标准和条件。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持转人工：UPF50+是可验证的产品性能指标，需要检测报告、执行标准和适用条件。；引用：无引用：系统因低于阈值转人工，未生成来源；性能真实性需检测材料支持。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统说明低于阈值并转人工，但没有指出应核验测试标准和条件。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM081</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款普通口香糖能够治愈牙周炎。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The claim suggests that a common chewing gum can cure periodontal disease, which is a strong health claim that is unsupported by evidence. Similar cases have shown that such health-related claims are considered illegal and misleading.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">支持：普通口香糖声称治愈牙周炎，属于明确的疾病治疗承诺。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分相关：来源案例涉及普通食品虚假保健功效，支持普通食品疾病治疗风险；不是口香糖或牙周炎同案。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">部分清楚：理由说明治愈疾病风险，但应明确引用只支持类别层面的判断。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">判断一致，引用部分支持</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持：普通口香糖声称治愈牙周炎，属于明确的疾病治疗承诺。；引用：部分相关：来源案例涉及普通食品虚假保健功效，支持普通食品疾病治疗风险；不是口香糖或牙周炎同案。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：部分清楚：理由说明治愈疾病风险，但应明确引用只支持类别层面的判断。；人工结论：当前证据更支持high_risk。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM084</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">穿上这款普通袜子就能百分之百预防静脉曲张。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；人工结论来自输入中的疾病预防和绝对保证表达。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚说明了转人工原因，但没有指出输入本身已含强疾病预防信号。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM086</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款空气净化器能去除99.9%的室内微尘。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">支持转人工：99.9%去除室内微尘是量化性能承诺，需要明确测试条件和检测报告。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；量化效果需产品检测材料支持。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统没有在证据不足时强行判断，但未提示检测环境、颗粒范围等关键条件。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持转人工：99.9%去除室内微尘是量化性能承诺，需要明确测试条件和检测报告。；引用：无引用：系统因低于阈值转人工，未生成来源；量化效果需产品检测材料支持。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统没有在证据不足时强行判断，但未提示检测环境、颗粒范围等关键条件。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM089</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">这款水壶获得了国际设计奖。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">支持转人工：获得国际设计奖是可核验事实，需要奖项名称、主办方和获奖证明。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；获奖真实性需外部材料核验。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚：系统说明证据不足并转人工，但未提示具体奖项核验路径。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">输入与判断：支持转人工：获得国际设计奖是可核验事实，需要奖项名称、主办方和获奖证明。；引用：无引用：系统因低于阈值转人工，未生成来源；获奖真实性需外部材料核验。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统说明证据不足并转人工，但未提示具体奖项核验路径。；人工结论：当前证据更支持evidence_needed。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">CLAIM090</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">这款家用靠垫保证治愈腰椎间盘突出。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">无引用：系统因低于阈值转人工，未生成来源；人工结论来自输入中的治愈保证。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">清楚说明了转人工原因，但没有指出输入本身已含强治愈信号。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">使用说明</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">用途</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">用于老师要求的20条人工复核记录。它是初筛质量检查，不是法律意见。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">样本</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">锁定测试集中的10条case_derived与10条synthetic；不包含开发集CLAIM072。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">标签边界</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">参考标签由项目人工编写，不是监管机关的官方标签；insufficient_evidence是系统转人工输出。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">引用核对</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">有引用的记录已对照对应政府页面；“部分支持”表示只能支持类别或类比风险，不能证明当前商家事实。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">建议检查</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">test_full.csv没有保存next_action，因此20条均只能如实标记为无法核查，不能补造建议。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">当前状态</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">禁止修改</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">不要修改参考标签、系统输出、锁定测试集或已有results文件来改善结果。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">低风险说明</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">low_risk仅表示未触发当前配置的风险，不等于法律批准；正式发布仍需人工确认。</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -658,12 +193,12 @@
     </x:font>
     <x:font>
       <x:sz val="9"/>
-      <x:name val="宋体"/>
+      <x:name val="Arial"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF222222"/>
-      <x:name val="微软雅黑"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="5">
@@ -836,7 +371,7 @@
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
-    <x:cellStyle name="常规" xfId="0"/>
+    <x:cellStyle name="Review body" xfId="0"/>
   </x:cellStyles>
   <x:dxfs count="3">
     <x:dxf>
@@ -880,25 +415,25 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManualReview20" displayName="ManualReview20" ref="A6:S26" totalsRowShown="0">
   <x:autoFilter ref="A6:S26"/>
   <x:tableColumns count="19">
-    <x:tableColumn id="1" name="序号"/>
+    <x:tableColumn id="1" name="No."/>
     <x:tableColumn id="2" name="claim_id"/>
-    <x:tableColumn id="3" name="中文文案"/>
-    <x:tableColumn id="4" name="样本类型"/>
-    <x:tableColumn id="5" name="参考标签"/>
-    <x:tableColumn id="6" name="系统输出"/>
-    <x:tableColumn id="7" name="转人工"/>
-    <x:tableColumn id="8" name="相似度"/>
-    <x:tableColumn id="9" name="模型理由"/>
-    <x:tableColumn id="10" name="输入与判断支持"/>
-    <x:tableColumn id="11" name="引用支持"/>
-    <x:tableColumn id="12" name="建议可执行性"/>
-    <x:tableColumn id="13" name="不确定性表达"/>
-    <x:tableColumn id="14" name="建议人工标签"/>
-    <x:tableColumn id="15" name="系统评价"/>
-    <x:tableColumn id="16" name="复核状态"/>
-    <x:tableColumn id="17" name="复核说明"/>
-    <x:tableColumn id="18" name="引用标题"/>
-    <x:tableColumn id="19" name="引用链接"/>
+    <x:tableColumn id="3" name="Claim (English translation)"/>
+    <x:tableColumn id="4" name="Sample type"/>
+    <x:tableColumn id="5" name="Reference label"/>
+    <x:tableColumn id="6" name="System output"/>
+    <x:tableColumn id="7" name="Abstained"/>
+    <x:tableColumn id="8" name="Top similarity"/>
+    <x:tableColumn id="9" name="Model reason"/>
+    <x:tableColumn id="10" name="Input and rating support"/>
+    <x:tableColumn id="11" name="Citation support"/>
+    <x:tableColumn id="12" name="Recommendation actionability"/>
+    <x:tableColumn id="13" name="Uncertainty wording"/>
+    <x:tableColumn id="14" name="Human label"/>
+    <x:tableColumn id="15" name="System assessment"/>
+    <x:tableColumn id="16" name="Review status"/>
+    <x:tableColumn id="17" name="Review conclusion"/>
+    <x:tableColumn id="18" name="Cited case (English summary title)"/>
+    <x:tableColumn id="19" name="Source URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1130,8 +665,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18.75">
-      <x:c r="A1" s="1" t="s">
-        <x:v>0</x:v>
+      <x:c r="A1" s="1" t="str">
+        <x:v>ClaimTrace: Manual review of 20 locked-test claims</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -1154,7 +689,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>10条案例改写 + 10条合成新文案。20条均已完成人工复核和结构化编码；复核结论不等于法律批准，正式发布仍需人工确认。</x:v>
+        <x:v>Ten case-derived and ten synthetic claims were reviewed. Coded results and source links appear below.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1197,40 +732,40 @@
       <x:c r="S3" s="2"/>
     </x:row>
     <x:row r="4" ht="13.899999618530273">
-      <x:c r="A4" s="4" t="s">
-        <x:v>1</x:v>
+      <x:c r="A4" s="4" t="str">
+        <x:v>Reviewed</x:v>
       </x:c>
       <x:c r="B4" s="5">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>2</x:v>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Case-derived</x:v>
       </x:c>
       <x:c r="D4" s="5">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>3</x:v>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Synthetic</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="s">
-        <x:v>4</x:v>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Abstentions</x:v>
       </x:c>
       <x:c r="H4" s="5" t="n">
         <x:f>COUNTIF(F7:F26,"insufficient_evidence")</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I4" s="5" t="s">
-        <x:v>5</x:v>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J4" s="5" t="n">
         <x:f>COUNTIF(Z7:Z26,"completed")</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K4" s="5" t="s">
-        <x:v>6</x:v>
+      <x:c r="K4" s="5" t="str">
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="L4" s="6" t="n">
         <x:f>COUNTIF(Z7:Z26,"pending")</x:f>
@@ -1266,62 +801,62 @@
       <x:c r="S5" s="2"/>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="7" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D6" s="7" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="K6" s="7" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="L6" s="7" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="M6" s="7" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="N6" s="7" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="O6" s="7" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="P6" s="7" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="Q6" s="7" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="R6" s="7" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="S6" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="A6" s="7" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="str">
+        <x:v>claim_id</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
+        <x:v>Claim (English translation)</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="str">
+        <x:v>Sample type</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="str">
+        <x:v>Reference label</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="str">
+        <x:v>System output</x:v>
+      </x:c>
+      <x:c r="G6" s="7" t="str">
+        <x:v>Abstained</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="str">
+        <x:v>Top similarity</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="str">
+        <x:v>Model reason</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="str">
+        <x:v>Input and rating support</x:v>
+      </x:c>
+      <x:c r="K6" s="7" t="str">
+        <x:v>Citation support</x:v>
+      </x:c>
+      <x:c r="L6" s="7" t="str">
+        <x:v>Recommendation actionability</x:v>
+      </x:c>
+      <x:c r="M6" s="7" t="str">
+        <x:v>Uncertainty wording</x:v>
+      </x:c>
+      <x:c r="N6" s="7" t="str">
+        <x:v>Human label</x:v>
+      </x:c>
+      <x:c r="O6" s="7" t="str">
+        <x:v>System assessment</x:v>
+      </x:c>
+      <x:c r="P6" s="7" t="str">
+        <x:v>Review status</x:v>
+      </x:c>
+      <x:c r="Q6" s="7" t="str">
+        <x:v>Review conclusion</x:v>
+      </x:c>
+      <x:c r="R6" s="7" t="str">
+        <x:v>Cited case (English summary title)</x:v>
+      </x:c>
+      <x:c r="S6" s="7" t="str">
+        <x:v>Source URL</x:v>
       </x:c>
       <x:c r="T6" s="19" t="str">
         <x:v>citation_present</x:v>
@@ -1350,58 +885,58 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="s">
-        <x:v>27</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>For only RMB 9 per month, this mobile data card provides unlimited high-speed data.</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G7" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H7" s="11">
         <x:v>0.46310000000000001</x:v>
       </x:c>
       <x:c r="I7" s="8" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="J7" s="8" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="K7" s="8" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="L7" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M7" s="8" t="s">
-        <x:v>36</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J7" s="8" t="str">
+        <x:v>Partial support: a low-priced unlimited data offer needs evidence of the tariff and allowance. A similar case alone does not establish that this offer is false.</x:v>
+      </x:c>
+      <x:c r="K7" s="8" t="str">
+        <x:v>Partial support: the official case found another company's CNY 9 per month data advertisement inconsistent with its actual offer. It supports a comparable risk, not a finding about this card.</x:v>
+      </x:c>
+      <x:c r="L7" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M7" s="8" t="str">
+        <x:v>Partly clear: the reason uses risk language, but the high_risk label blurs analogy with facts about this seller.</x:v>
       </x:c>
       <x:c r="N7" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O7" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="str">
+        <x:v>Overclassified: the reference label calls for evidence, while the system assigns high risk.</x:v>
       </x:c>
       <x:c r="P7" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q7" s="8" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="R7" s="8" t="s">
-        <x:v>39</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q7" s="8" t="str">
+        <x:v>Human review favors evidence_needed until the current price and data terms are verified.</x:v>
+      </x:c>
+      <x:c r="R7" s="8" t="str">
+        <x:v>Beijing: misleading mobile-data plan pricing</x:v>
       </x:c>
       <x:c r="S7" s="8" t="s">
-        <x:v>40</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T7" s="21" t="str">
         <x:v>yes</x:v>
@@ -1430,58 +965,58 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B8" s="9" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="s">
-        <x:v>42</x:v>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>Using this skincare set for seven days will completely eliminate redness, itching and acne.</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F8" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G8" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H8" s="11">
         <x:v>0.41060000000000002</x:v>
       </x:c>
       <x:c r="I8" s="8" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="J8" s="8" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="K8" s="8" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="L8" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M8" s="8" t="s">
-        <x:v>46</x:v>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J8" s="8" t="str">
+        <x:v>Supported: a promise to completely eliminate several skin symptoms within seven days is an explicit, absolute treatment-effect claim.</x:v>
+      </x:c>
+      <x:c r="K8" s="8" t="str">
+        <x:v>Directly relevant: the official case concerns a cosmetic advertised as treating redness, itching, stinging and acne. The product type and symptoms closely match.</x:v>
+      </x:c>
+      <x:c r="L8" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M8" s="8" t="str">
+        <x:v>Partly clear: the reason explains the similar case and medicine-confusion risk, but does not explicitly call for checking this product's facts before publication.</x:v>
       </x:c>
       <x:c r="N8" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O8" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="str">
+        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q8" s="8" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="R8" s="8" t="s">
-        <x:v>49</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q8" s="8" t="str">
+        <x:v>Human review agrees with high_risk because the claim guarantees treatment of skin symptoms.</x:v>
+      </x:c>
+      <x:c r="R8" s="8" t="str">
+        <x:v>Hangzhou: cosmetic advertised as treating skin conditions</x:v>
       </x:c>
       <x:c r="S8" s="8" t="s">
-        <x:v>40</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T8" s="21" t="str">
         <x:v>yes</x:v>
@@ -1510,58 +1045,58 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="9" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="C9" s="8" t="s">
-        <x:v>51</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>A large number of consumers have personally confirmed that this jelly produces rapid weight loss.</x:v>
       </x:c>
       <x:c r="D9" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H9" s="11">
         <x:v>0.48559999999999998</x:v>
       </x:c>
       <x:c r="I9" s="8" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="J9" s="8" t="s">
-        <x:v>53</x:v>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J9" s="8" t="str">
+        <x:v>Partial support: rapid weight loss and claimed consumer confirmation need efficacy evidence and authentic reviews. The wording alone does not establish falsity.</x:v>
       </x:c>
       <x:c r="K9" s="8" t="str">
-        <x:v>弱相关且引用与理由不完全匹配：当前链接指向汕尾普通食品功效案例，页面未包含果冻减肥或虚假用户评论内容，只能提供普通食品功效宣传的类别层面支持。</x:v>
-      </x:c>
-      <x:c r="L9" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M9" s="8" t="s">
-        <x:v>54</x:v>
+        <x:v>Weak match: the linked Shanwei case concerns efficacy claims for ordinary food, not jelly weight loss or fabricated user comments. It offers category-level context only.</x:v>
+      </x:c>
+      <x:c r="L9" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M9" s="8" t="str">
+        <x:v>Insufficient: the reason treats missing evidence as high risk without explaining that the current reviews and product effects still need verification.</x:v>
       </x:c>
       <x:c r="N9" s="10" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O9" s="10" t="str">
-        <x:v>过度升级，且当前引用与模型理由不完全匹配</x:v>
+        <x:v>Overclassified: the citation does not fully support the model's stated reason.</x:v>
       </x:c>
       <x:c r="P9" s="10" t="str">
-        <x:v>已确认</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="Q9" s="8" t="str">
-        <x:v>输入与判断：部分支持：快速减肥和“消费者证明”需要效果证据及评价真实性证明，尚不能仅凭文案认定虚假。；引用：弱相关且引用与理由不完全匹配：当前链接指向汕尾普通食品功效案例，页面未包含果冻减肥或虚假用户评论内容，只能提供普通食品功效宣传的类别层面支持。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：不足：理由将缺少证据直接推向高风险，没有充分说明仍需核验当前评价和产品效果。；人工结论：当前证据更支持evidence_needed。</x:v>
-      </x:c>
-      <x:c r="R9" s="8" t="s">
-        <x:v>55</x:v>
+        <x:v>Human review favors evidence_needed; the cited case does not establish this product's results or review authenticity.</x:v>
+      </x:c>
+      <x:c r="R9" s="8" t="str">
+        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
       </x:c>
       <x:c r="S9" s="8" t="s">
-        <x:v>56</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T9" s="21" t="str">
         <x:v>yes</x:v>
@@ -1590,58 +1125,58 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B10" s="9" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C10" s="8" t="s">
-        <x:v>58</x:v>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>Testing proves that this home beauty device can significantly improve skin firmness.</x:v>
       </x:c>
       <x:c r="D10" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G10" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H10" s="11">
         <x:v>0.45450000000000002</x:v>
       </x:c>
       <x:c r="I10" s="8" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="J10" s="8" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="K10" s="8" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="L10" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M10" s="8" t="s">
-        <x:v>62</x:v>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J10" s="8" t="str">
+        <x:v>Partial support: improved skin firmness is a testable efficacy claim needing test evidence. The submitted wording alone does not establish high risk.</x:v>
+      </x:c>
+      <x:c r="K10" s="8" t="str">
+        <x:v>Weak match: the source concerns false whitening claims for ordinary hand soap, not a beauty device or skin-firmness performance.</x:v>
+      </x:c>
+      <x:c r="L10" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M10" s="8" t="str">
+        <x:v>Insufficient: the reason frames firmness as a treatment promise without addressing product type or the missing performance evidence.</x:v>
       </x:c>
       <x:c r="N10" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O10" s="10" t="s">
-        <x:v>63</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="str">
+        <x:v>Overclassified, with a weak citation.</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q10" s="8" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="R10" s="8" t="s">
-        <x:v>65</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q10" s="8" t="str">
+        <x:v>Human review favors evidence_needed until the claimed test and performance evidence are checked.</x:v>
+      </x:c>
+      <x:c r="R10" s="8" t="str">
+        <x:v>Fangxian: unsupported whitening claim for hand wash</x:v>
       </x:c>
       <x:c r="S10" s="8" t="s">
-        <x:v>66</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="T10" s="21" t="str">
         <x:v>yes</x:v>
@@ -1670,58 +1205,58 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B11" s="9" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="C11" s="8" t="s">
-        <x:v>68</x:v>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>This ordinary paste can repair physical damage and relieve disease-related symptoms.</x:v>
       </x:c>
       <x:c r="D11" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H11" s="11">
         <x:v>0.31209999999999999</x:v>
       </x:c>
       <x:c r="I11" s="8" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="J11" s="8" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="K11" s="8" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="L11" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M11" s="8" t="s">
-        <x:v>72</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J11" s="8" t="str">
+        <x:v>Supported: an ordinary paste claiming to repair physical damage and relieve disease symptoms makes an explicit treatment-effect claim.</x:v>
+      </x:c>
+      <x:c r="K11" s="8" t="str">
+        <x:v>Directly relevant: the official case concerns an ordinary paste promoted through disease-treatment and restored-mobility claims.</x:v>
+      </x:c>
+      <x:c r="L11" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M11" s="8" t="str">
+        <x:v>Partly clear: the reason explains the medical wording risk, but the final publication decision still requires checking the product facts.</x:v>
       </x:c>
       <x:c r="N11" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O11" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O11" s="10" t="str">
+        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
       </x:c>
       <x:c r="P11" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q11" s="8" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="R11" s="8" t="s">
-        <x:v>74</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q11" s="8" t="str">
+        <x:v>Human review agrees with high_risk because an ordinary paste is presented as treating disease symptoms.</x:v>
+      </x:c>
+      <x:c r="R11" s="8" t="str">
+        <x:v>Qingdao: treatment claims for an ordinary ointment</x:v>
       </x:c>
       <x:c r="S11" s="8" t="s">
-        <x:v>75</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T11" s="21" t="str">
         <x:v>yes</x:v>
@@ -1750,58 +1285,58 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B12" s="9" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="C12" s="8" t="s">
-        <x:v>77</x:v>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>This product can comprehensively improve bodily functions and performs far better than comparable products.</x:v>
       </x:c>
       <x:c r="D12" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F12" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G12" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H12" s="11">
         <x:v>0.36980000000000002</x:v>
       </x:c>
       <x:c r="I12" s="8" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="J12" s="8" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="K12" s="8" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="L12" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M12" s="8" t="s">
-        <x:v>81</x:v>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J12" s="8" t="str">
+        <x:v>Partial support: broad claims of improved bodily function and superiority to comparable products need evidence. The input alone does not establish high risk.</x:v>
+      </x:c>
+      <x:c r="K12" s="8" t="str">
+        <x:v>Partly relevant: the source concerns false health or improvement claims for ordinary food, but not the same broad bodily-function claim.</x:v>
+      </x:c>
+      <x:c r="L12" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M12" s="8" t="str">
+        <x:v>Insufficient: the reason cites a lack of scientific support without first calling for product and comparison evidence.</x:v>
       </x:c>
       <x:c r="N12" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O12" s="10" t="s">
-        <x:v>82</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O12" s="10" t="str">
+        <x:v>Overclassified: requesting supporting evidence fits the reference label better.</x:v>
       </x:c>
       <x:c r="P12" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q12" s="8" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="R12" s="8" t="s">
-        <x:v>55</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q12" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the performance and comparative claims.</x:v>
+      </x:c>
+      <x:c r="R12" s="8" t="str">
+        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
       </x:c>
       <x:c r="S12" s="8" t="s">
-        <x:v>56</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T12" s="21" t="str">
         <x:v>yes</x:v>
@@ -1830,58 +1365,58 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B13" s="9" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C13" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>All pearls sold by this store are natural and are supplied with genuine authoritative certificates.</x:v>
       </x:c>
       <x:c r="D13" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G13" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H13" s="11">
         <x:v>0.73229999999999995</x:v>
       </x:c>
       <x:c r="I13" s="8" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="J13" s="8" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="K13" s="8" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="L13" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M13" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J13" s="8" t="str">
+        <x:v>Partial support: natural pearls and authoritative certificates are authenticity claims requiring this store's appraisal and certificate records.</x:v>
+      </x:c>
+      <x:c r="K13" s="8" t="str">
+        <x:v>Highly relevant, but not direct proof: the official case involved imitation pearls and forged certificates. It supports verification, not an allegation about this store.</x:v>
+      </x:c>
+      <x:c r="L13" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M13" s="8" t="str">
+        <x:v>Insufficient: the reason moves from an earlier seller's conduct to concern about the current goods without clearly separating the two.</x:v>
       </x:c>
       <x:c r="N13" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O13" s="10" t="s">
-        <x:v>90</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="str">
+        <x:v>Overclassified: analogous risk does not establish the current facts.</x:v>
       </x:c>
       <x:c r="P13" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q13" s="8" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="R13" s="8" t="s">
-        <x:v>92</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q13" s="8" t="str">
+        <x:v>Human review favors evidence_needed pending appraisal and certificate checks.</x:v>
+      </x:c>
+      <x:c r="R13" s="8" t="str">
+        <x:v>Zhuji: imitation pearls sold as genuine</x:v>
       </x:c>
       <x:c r="S13" s="8" t="s">
-        <x:v>75</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T13" s="21" t="str">
         <x:v>yes</x:v>
@@ -1910,52 +1445,52 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="9" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="C14" s="8" t="s">
-        <x:v>94</x:v>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>All Hetian jade sold in the livestream comes from the mine shown by the host and has a completely reliable origin.</x:v>
       </x:c>
       <x:c r="D14" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F14" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G14" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H14" s="11">
         <x:v>0.2928</x:v>
       </x:c>
       <x:c r="I14" s="8" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="J14" s="8" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="K14" s="8" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="L14" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M14" s="8" t="s">
-        <x:v>100</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J14" s="8" t="str">
+        <x:v>Human review is supported: the mine-origin and completely reliable provenance claims need supply-chain and origin records; abstention fits the low retrieval score.</x:v>
+      </x:c>
+      <x:c r="K14" s="8" t="str">
+        <x:v>No citation: the 0.2928 similarity score is below the provisional 0.30 threshold, so the system returned no source.</x:v>
+      </x:c>
+      <x:c r="L14" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M14" s="8" t="str">
+        <x:v>Clear about the threshold and human review, but it does not identify the origin and supply-chain records to check.</x:v>
       </x:c>
       <x:c r="N14" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O14" s="10" t="s">
-        <x:v>101</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O14" s="10" t="str">
+        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
       </x:c>
       <x:c r="P14" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q14" s="8" t="s">
-        <x:v>102</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q14" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the jade-origin claim.</x:v>
       </x:c>
       <x:c r="R14" s="8"/>
       <x:c r="S14" s="8"/>
@@ -1986,58 +1521,58 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B15" s="9" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="s">
-        <x:v>104</x:v>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>Authoritative research and genuine user feedback prove that royal jelly has pharmacological effects including anti-tumour activity.</x:v>
       </x:c>
       <x:c r="D15" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F15" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G15" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H15" s="11">
         <x:v>0.43120000000000003</x:v>
       </x:c>
       <x:c r="I15" s="8" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="J15" s="8" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="K15" s="8" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="L15" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M15" s="8" t="s">
-        <x:v>108</x:v>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="J15" s="8" t="str">
+        <x:v>Supported: attributing anti-tumour pharmacological effects to an ordinary bee product is an explicit disease-treatment or drug-effect claim.</x:v>
+      </x:c>
+      <x:c r="K15" s="8" t="str">
+        <x:v>Directly relevant: the official case addresses royal jelly, pharmacological effects, user feedback and research-body claims closely matching this input.</x:v>
+      </x:c>
+      <x:c r="L15" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M15" s="8" t="str">
+        <x:v>Partly clear: the reason identifies the medical claim, while the precise product and advertising context still need checking.</x:v>
       </x:c>
       <x:c r="N15" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O15" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O15" s="10" t="str">
+        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
       </x:c>
       <x:c r="P15" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q15" s="8" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="R15" s="8" t="s">
-        <x:v>110</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q15" s="8" t="str">
+        <x:v>Human review agrees with high_risk because ordinary royal jelly is presented as having pharmacological effects.</x:v>
+      </x:c>
+      <x:c r="R15" s="8" t="str">
+        <x:v>Qiandaohu Chunxin: false royal-jelly claims</x:v>
       </x:c>
       <x:c r="S15" s="8" t="s">
-        <x:v>111</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="T15" s="21" t="str">
         <x:v>yes</x:v>
@@ -2066,58 +1601,58 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B16" s="9" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="s">
-        <x:v>113</x:v>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>Drinking this camel milk powder every day can effectively control blood sugar and other related chronic health conditions.</x:v>
       </x:c>
       <x:c r="D16" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F16" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G16" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H16" s="11">
         <x:v>0.68120000000000003</x:v>
       </x:c>
       <x:c r="I16" s="8" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="J16" s="8" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="K16" s="8" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="L16" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M16" s="8" t="s">
-        <x:v>117</x:v>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="J16" s="8" t="str">
+        <x:v>Supported: ordinary food advertised as controlling blood sugar and related chronic conditions makes a disease-prevention or treatment claim.</x:v>
+      </x:c>
+      <x:c r="K16" s="8" t="str">
+        <x:v>Directly relevant: the official case involves camel milk powder advertised as lowering blood sugar and addressing the same conditions.</x:v>
+      </x:c>
+      <x:c r="L16" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M16" s="8" t="str">
+        <x:v>Partly clear: the reason identifies the disease claim, while final review still needs the product type and complete advertising context.</x:v>
       </x:c>
       <x:c r="N16" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O16" s="10" t="s">
-        <x:v>47</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O16" s="10" t="str">
+        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
       </x:c>
       <x:c r="P16" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q16" s="8" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="R16" s="8" t="s">
-        <x:v>119</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q16" s="8" t="str">
+        <x:v>Human review agrees with high_risk because the milk powder is promoted for chronic conditions.</x:v>
+      </x:c>
+      <x:c r="R16" s="8" t="str">
+        <x:v>Yunnan Xinghao: disease claims for camel milk powder</x:v>
       </x:c>
       <x:c r="S16" s="8" t="s">
-        <x:v>111</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="T16" s="21" t="str">
         <x:v>yes</x:v>
@@ -2146,52 +1681,52 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="9" t="s">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="s">
-        <x:v>121</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>This notebook is available with lined or blank pages.</x:v>
       </x:c>
       <x:c r="D17" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E17" s="9" t="s">
-        <x:v>123</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F17" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H17" s="11">
         <x:v>0.11409999999999999</x:v>
       </x:c>
       <x:c r="I17" s="8" t="s">
-        <x:v>97</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str">
-        <x:v>支持低风险：仅描述笔记本页面规格，不涉及已配置的高风险类型；按当前阈值转人工符合系统规则，但会降低低风险样本的覆盖率。</x:v>
-      </x:c>
-      <x:c r="K17" s="8" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="L17" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M17" s="8" t="s">
-        <x:v>125</x:v>
+        <x:v>Low risk under the configured checks: this describes notebook page options. Threshold-based abstention nevertheless reduces coverage of ordinary product descriptions.</x:v>
+      </x:c>
+      <x:c r="K17" s="8" t="str">
+        <x:v>No citation: the system abstained below the threshold. The input itself supports the limited low-risk reference label.</x:v>
+      </x:c>
+      <x:c r="L17" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M17" s="8" t="str">
+        <x:v>Clear about abstention, but the system does not distinguish a routine specification from a potentially risky claim.</x:v>
       </x:c>
       <x:c r="N17" s="10" t="s">
-        <x:v>123</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="O17" s="10" t="str">
-        <x:v>按当前阈值转人工合理，但低风险样本未被系统覆盖</x:v>
+        <x:v>Abstention follows the current threshold rule, but this low-risk item is not covered.</x:v>
       </x:c>
       <x:c r="P17" s="10" t="str">
-        <x:v>已确认</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="Q17" s="8" t="str">
-        <x:v>输入与判断：支持低风险：仅描述笔记本页面规格，不涉及已配置的高风险类型；按当前阈值转人工符合系统规则，但会降低低风险样本的覆盖率。；引用：无引用：系统因低于阈值转人工，未生成来源；低风险判断仅基于输入内容，不等于法律批准。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚：系统说明低于阈值并转人工，但没有区分普通商品规格信息。；人工结论：当前证据更支持low_risk。</x:v>
+        <x:v>Human review favors low_risk for the page-format description.</x:v>
       </x:c>
       <x:c r="R17" s="8"/>
       <x:c r="S17" s="8"/>
@@ -2222,52 +1757,52 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B18" s="9" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="s">
-        <x:v>127</x:v>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>This Bluetooth speaker sold more than one million units in one year.</x:v>
       </x:c>
       <x:c r="D18" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E18" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F18" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G18" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H18" s="11">
         <x:v>0.2661</x:v>
       </x:c>
       <x:c r="I18" s="8" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="J18" s="8" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="K18" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="L18" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M18" s="8" t="s">
-        <x:v>130</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J18" s="8" t="str">
+        <x:v>Human review is supported: more than one million annual sales is a verifiable claim needing platform, order or sales records.</x:v>
+      </x:c>
+      <x:c r="K18" s="8" t="str">
+        <x:v>No citation: the system abstained below the threshold; the sales count needs independent records.</x:v>
+      </x:c>
+      <x:c r="L18" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M18" s="8" t="str">
+        <x:v>Clear about insufficient retrieval evidence, but it does not identify which sales records to check.</x:v>
       </x:c>
       <x:c r="N18" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O18" s="10" t="s">
-        <x:v>101</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O18" s="10" t="str">
+        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
       </x:c>
       <x:c r="P18" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q18" s="8" t="s">
-        <x:v>131</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q18" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the annual sales figure.</x:v>
       </x:c>
       <x:c r="R18" s="8"/>
       <x:c r="S18" s="8"/>
@@ -2298,58 +1833,58 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B19" s="9" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="s">
-        <x:v>133</x:v>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>This ordinary milk drink can treat anaemia.</x:v>
       </x:c>
       <x:c r="D19" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E19" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F19" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G19" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H19" s="11">
         <x:v>0.49709999999999999</x:v>
       </x:c>
       <x:c r="I19" s="8" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="J19" s="8" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="K19" s="8" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="L19" s="8" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="J19" s="8" t="str">
+        <x:v>Supported: an ordinary milk drink advertised as treating anaemia makes an explicit disease-treatment claim.</x:v>
+      </x:c>
+      <x:c r="K19" s="8" t="str">
+        <x:v>Partly relevant: the cited case concerns disease-related claims for ordinary food, but not anaemia or this milk drink.</x:v>
+      </x:c>
+      <x:c r="L19" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M19" s="8" t="str">
+        <x:v>Partly clear: the reason identifies the treatment risk, but wording that a similar case proves wrongdoing could imply a conclusion about this product.</x:v>
+      </x:c>
+      <x:c r="N19" s="10" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="str">
+        <x:v>The system label matches the human label; the citation supports the category-level risk.</x:v>
+      </x:c>
+      <x:c r="P19" s="10" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q19" s="8" t="str">
+        <x:v>Human review agrees with high_risk for the anaemia-treatment wording.</x:v>
+      </x:c>
+      <x:c r="R19" s="8" t="str">
+        <x:v>Chengmai Hengsheng Hospital: health claims for beverage powder</x:v>
+      </x:c>
+      <x:c r="S19" s="8" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="M19" s="8" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="N19" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O19" s="10" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="P19" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q19" s="8" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="R19" s="8" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="S19" s="8" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="T19" s="21" t="str">
         <x:v>yes</x:v>
@@ -2378,52 +1913,52 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B20" s="9" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="C20" s="8" t="s">
-        <x:v>143</x:v>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>This umbrella is available in yellow and black.</x:v>
       </x:c>
       <x:c r="D20" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E20" s="9" t="s">
-        <x:v>123</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F20" s="9" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G20" s="9" t="s">
         <x:v>31</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H20" s="11">
         <x:v>0.34699999999999998</x:v>
       </x:c>
       <x:c r="I20" s="8" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="J20" s="8" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="K20" s="8" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="L20" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M20" s="8" t="s">
-        <x:v>147</x:v>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="J20" s="8" t="str">
+        <x:v>Supported: the claim only lists umbrella colour options and triggers no configured risk; the listing should still match the goods.</x:v>
+      </x:c>
+      <x:c r="K20" s="8" t="str">
+        <x:v>No citation: the colour description can be checked against the goods, and this low-risk result does not require a case citation.</x:v>
+      </x:c>
+      <x:c r="L20" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M20" s="8" t="str">
+        <x:v>Mostly clear: the model states that no configured risk was found and does not present the result as approval.</x:v>
       </x:c>
       <x:c r="N20" s="10" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="O20" s="10" t="s">
-        <x:v>148</x:v>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="O20" s="10" t="str">
+        <x:v>The system label matches the human label; no citation is acceptable here.</x:v>
       </x:c>
       <x:c r="P20" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q20" s="8" t="s">
-        <x:v>149</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q20" s="8" t="str">
+        <x:v>Human review agrees with low_risk for the colour-options description.</x:v>
       </x:c>
       <x:c r="R20" s="8"/>
       <x:c r="S20" s="8"/>
@@ -2454,52 +1989,52 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B21" s="9" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="C21" s="8" t="s">
-        <x:v>151</x:v>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>This sun-protective jacket has a UPF rating of 50+.</x:v>
       </x:c>
       <x:c r="D21" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E21" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F21" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H21" s="11">
         <x:v>0.26019999999999999</x:v>
       </x:c>
       <x:c r="I21" s="8" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="J21" s="8" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="K21" s="8" t="s">
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="L21" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M21" s="8" t="s">
-        <x:v>154</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J21" s="8" t="str">
+        <x:v>Human review is supported: UPF 50+ is a testable performance rating needing a test report, standard and applicable conditions.</x:v>
+      </x:c>
+      <x:c r="K21" s="8" t="str">
+        <x:v>No citation: the system abstained below the threshold; the rating needs product testing records.</x:v>
+      </x:c>
+      <x:c r="L21" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M21" s="8" t="str">
+        <x:v>Clear about abstention, but it does not identify the test standard or conditions to verify.</x:v>
       </x:c>
       <x:c r="N21" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O21" s="10" t="s">
-        <x:v>101</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="str">
+        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
       </x:c>
       <x:c r="P21" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q21" s="8" t="s">
-        <x:v>155</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q21" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the UPF rating.</x:v>
       </x:c>
       <x:c r="R21" s="8"/>
       <x:c r="S21" s="8"/>
@@ -2530,58 +2065,58 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B22" s="9" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="C22" s="8" t="s">
-        <x:v>157</x:v>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>This ordinary chewing gum can cure periodontitis.</x:v>
       </x:c>
       <x:c r="D22" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E22" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F22" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G22" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H22" s="11">
         <x:v>0.42049999999999998</x:v>
       </x:c>
       <x:c r="I22" s="8" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="J22" s="8" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="K22" s="8" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="L22" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M22" s="8" t="s">
-        <x:v>161</x:v>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J22" s="8" t="str">
+        <x:v>Supported: ordinary chewing gum claiming to cure periodontitis makes an explicit disease-treatment promise.</x:v>
+      </x:c>
+      <x:c r="K22" s="8" t="str">
+        <x:v>Partly relevant: the source concerns unsupported health effects for ordinary food, not chewing gum or periodontitis.</x:v>
+      </x:c>
+      <x:c r="L22" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M22" s="8" t="str">
+        <x:v>Partly clear: the reason identifies the cure claim, but should state that the citation supports only category-level context.</x:v>
       </x:c>
       <x:c r="N22" s="10" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="O22" s="10" t="s">
-        <x:v>162</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O22" s="10" t="str">
+        <x:v>The system label matches the human label; the citation provides partial support.</x:v>
       </x:c>
       <x:c r="P22" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q22" s="8" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="R22" s="8" t="s">
-        <x:v>55</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q22" s="8" t="str">
+        <x:v>Human review agrees with high_risk because the gum is advertised as curing a disease.</x:v>
+      </x:c>
+      <x:c r="R22" s="8" t="str">
+        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
       </x:c>
       <x:c r="S22" s="8" t="s">
-        <x:v>56</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T22" s="21" t="str">
         <x:v>yes</x:v>
@@ -2610,52 +2145,52 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="9" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="C23" s="8" t="s">
-        <x:v>165</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>Wearing these ordinary socks will prevent varicose veins with 100% certainty.</x:v>
       </x:c>
       <x:c r="D23" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E23" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H23" s="11">
         <x:v>0.28810000000000002</x:v>
       </x:c>
       <x:c r="I23" s="8" t="s">
-        <x:v>97</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J23" s="8" t="str">
-        <x:v>转人工符合当前阈值机制，但规则未优先识别明显风险：普通袜子“百分之百预防”疾病属于强绝对化疾病预防承诺，人工应判高风险。</x:v>
-      </x:c>
-      <x:c r="K23" s="8" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="L23" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M23" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>Abstention follows the threshold rule, but it misses an obvious signal: ordinary socks promising 100% prevention of varicose veins make an absolute disease-prevention claim.</x:v>
+      </x:c>
+      <x:c r="K23" s="8" t="str">
+        <x:v>No citation: retrieval was below the threshold. The human label follows from the disease-prevention and absolute-guarantee wording.</x:v>
+      </x:c>
+      <x:c r="L23" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M23" s="8" t="str">
+        <x:v>Clear about why the system abstained, but it does not flag the strong prevention claim already present in the input.</x:v>
       </x:c>
       <x:c r="N23" s="10" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O23" s="10" t="str">
-        <x:v>转人工符合当前阈值机制，但规则未优先识别疾病预防和绝对保证表达</x:v>
+        <x:v>Abstention follows the threshold rule, but the rules miss disease prevention and an absolute guarantee.</x:v>
       </x:c>
       <x:c r="P23" s="10" t="str">
-        <x:v>已确认</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="Q23" s="8" t="str">
-        <x:v>输入与判断：转人工符合当前阈值机制，但规则未优先识别明显风险：普通袜子“百分之百预防”疾病属于强绝对化疾病预防承诺，人工应判高风险。；引用：无引用：系统因低于阈值转人工，未生成来源；人工结论来自输入中的疾病预防和绝对保证表达。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚说明了转人工原因，但没有指出输入本身已含强疾病预防信号。；人工结论：当前证据更支持high_risk。</x:v>
+        <x:v>Human review favors high_risk for the 100% disease-prevention promise.</x:v>
       </x:c>
       <x:c r="R23" s="8"/>
       <x:c r="S23" s="8"/>
@@ -2686,52 +2221,52 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B24" s="9" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="C24" s="8" t="s">
-        <x:v>169</x:v>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="str">
+        <x:v>This air purifier removes 99.9% of fine indoor dust.</x:v>
       </x:c>
       <x:c r="D24" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E24" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F24" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G24" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H24" s="11">
         <x:v>0.29170000000000001</x:v>
       </x:c>
       <x:c r="I24" s="8" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="J24" s="8" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="K24" s="8" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="L24" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M24" s="8" t="s">
-        <x:v>172</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J24" s="8" t="str">
+        <x:v>Human review is supported: a 99.9% indoor dust-removal claim needs defined test conditions and a performance report.</x:v>
+      </x:c>
+      <x:c r="K24" s="8" t="str">
+        <x:v>No citation: the system abstained below the threshold; quantified efficacy needs product-test evidence.</x:v>
+      </x:c>
+      <x:c r="L24" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M24" s="8" t="str">
+        <x:v>Clear about abstention, but it does not identify the test environment or particle range.</x:v>
       </x:c>
       <x:c r="N24" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O24" s="10" t="s">
-        <x:v>101</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O24" s="10" t="str">
+        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
       </x:c>
       <x:c r="P24" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q24" s="8" t="s">
-        <x:v>173</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q24" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the quantified removal claim.</x:v>
       </x:c>
       <x:c r="R24" s="8"/>
       <x:c r="S24" s="8"/>
@@ -2762,52 +2297,52 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B25" s="9" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C25" s="8" t="s">
-        <x:v>175</x:v>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C25" s="8" t="str">
+        <x:v>This water bottle received an international design award.</x:v>
       </x:c>
       <x:c r="D25" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E25" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F25" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G25" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H25" s="11">
         <x:v>0.28570000000000001</x:v>
       </x:c>
       <x:c r="I25" s="8" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="J25" s="8" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="K25" s="8" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="L25" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M25" s="8" t="s">
-        <x:v>178</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J25" s="8" t="str">
+        <x:v>Human review is supported: an international design award is a verifiable fact needing the award name, organiser and winner record.</x:v>
+      </x:c>
+      <x:c r="K25" s="8" t="str">
+        <x:v>No citation: the system abstained below the threshold; award authenticity needs an external record.</x:v>
+      </x:c>
+      <x:c r="L25" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M25" s="8" t="str">
+        <x:v>Clear about abstention, but it does not point to the specific award record to check.</x:v>
       </x:c>
       <x:c r="N25" s="10" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="O25" s="10" t="s">
-        <x:v>101</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="str">
+        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
       </x:c>
       <x:c r="P25" s="10" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="Q25" s="8" t="s">
-        <x:v>179</x:v>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="Q25" s="8" t="str">
+        <x:v>Human review favors evidence_needed for the award claim.</x:v>
       </x:c>
       <x:c r="R25" s="8"/>
       <x:c r="S25" s="8"/>
@@ -2838,52 +2373,52 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B26" s="9" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="C26" s="8" t="s">
-        <x:v>181</x:v>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C26" s="8" t="str">
+        <x:v>This household cushion guarantees a cure for a herniated lumbar disc.</x:v>
       </x:c>
       <x:c r="D26" s="9" t="s">
-        <x:v>122</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E26" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F26" s="9" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="G26" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H26" s="11">
         <x:v>0.17299999999999999</x:v>
       </x:c>
       <x:c r="I26" s="8" t="s">
-        <x:v>97</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J26" s="8" t="str">
-        <x:v>转人工符合当前阈值机制，但规则未优先识别明显风险：家用靠垫“保证治愈”疾病属于强治疗承诺，人工应判高风险。</x:v>
-      </x:c>
-      <x:c r="K26" s="8" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="L26" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M26" s="8" t="s">
-        <x:v>183</x:v>
+        <x:v>Abstention follows the threshold rule, but it misses an obvious signal: a household cushion promising a cure for a herniated disc makes a strong treatment claim.</x:v>
+      </x:c>
+      <x:c r="K26" s="8" t="str">
+        <x:v>No citation: retrieval was below the threshold. The human label follows from the guaranteed-cure wording in the input.</x:v>
+      </x:c>
+      <x:c r="L26" s="8" t="str">
+        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
+      </x:c>
+      <x:c r="M26" s="8" t="str">
+        <x:v>Clear about why the system abstained, but it does not flag the cure guarantee already present in the input.</x:v>
       </x:c>
       <x:c r="N26" s="10" t="s">
-        <x:v>30</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O26" s="10" t="str">
-        <x:v>转人工符合当前阈值机制，但规则未优先识别明显的治愈保证</x:v>
+        <x:v>Abstention follows the threshold rule, but the rules miss the explicit cure guarantee.</x:v>
       </x:c>
       <x:c r="P26" s="10" t="str">
-        <x:v>已确认</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="Q26" s="8" t="str">
-        <x:v>输入与判断：转人工符合当前阈值机制，但规则未优先识别明显风险：家用靠垫“保证治愈”疾病属于强治疗承诺，人工应判高风险。；引用：无引用：系统因低于阈值转人工，未生成来源；人工结论来自输入中的治愈保证。；建议可执行性：无法核查：test_full.csv未保存next_action字段。；不确定性：清楚说明了转人工原因，但没有指出输入本身已含强治愈信号。；人工结论：当前证据更支持high_risk。</x:v>
+        <x:v>Human review favors high_risk for the guaranteed cure.</x:v>
       </x:c>
       <x:c r="R26" s="8"/>
       <x:c r="S26" s="8"/>
@@ -2911,13 +2446,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="P7:P26">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="已确认"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="待确认"/>
-    <x:cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="需修改"/>
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Completed"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Pending"/>
+    <x:cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Needs revision"/>
   </x:conditionalFormatting>
   <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="P7:P26">
-      <x:formula1>"待确认,已确认,需修改"</x:formula1>
+      <x:formula1>"Completed,Pending,Needs revision"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="T7:T26">
       <x:formula1>"yes,no,uncertain"</x:formula1>
@@ -2940,7 +2475,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e20956d4a224274"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78fa3220e44f4c5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2957,8 +2492,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18.75">
-      <x:c r="A1" s="1" t="s">
-        <x:v>184</x:v>
+      <x:c r="A1" s="1" t="str">
+        <x:v>Review notes</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
     </x:row>
@@ -2967,75 +2502,75 @@
       <x:c r="B2" s="2"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="15" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="s">
-        <x:v>186</x:v>
+      <x:c r="A3" s="15" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>Manual quality review of 20 locked-test results.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="16" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="s">
-        <x:v>188</x:v>
+      <x:c r="A4" s="16" t="str">
+        <x:v>Sample</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="str">
+        <x:v>Ten case-derived and ten synthetic test claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="16" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="B5" s="13" t="s">
-        <x:v>190</x:v>
+      <x:c r="A5" s="16" t="str">
+        <x:v>Reference labels</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="str">
+        <x:v>Project-defined labels support comparison. insufficient_evidence is an abstention, not a reference label.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="16" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="B6" s="13" t="s">
-        <x:v>192</x:v>
+      <x:c r="A6" s="16" t="str">
+        <x:v>Citation checks</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="str">
+        <x:v>Present citations were checked against source pages. Partial support indicates comparable risk, not a finding about the current seller.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="16" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="B7" s="13" t="s">
-        <x:v>194</x:v>
+      <x:c r="A7" s="16" t="str">
+        <x:v>Actionability</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="str">
+        <x:v>Historical test_full.csv lacks next_action; actionability is not_applicable for all 20 reviews.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>结构化字段</x:v>
+        <x:v>Coded fields</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>复核记录T至Z列保存结构化结果。citation_supported、reason_supported和uncertainty_clear基于已确认的人工复核结论；无引用记录的citation_supported记为not_applicable。</x:v>
+        <x:v>Columns T-Z retain the structured review codes. A missing citation is coded not_applicable for citation_supported.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="16" t="s">
-        <x:v>195</x:v>
+      <x:c r="A9" s="16" t="str">
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>20条记录均已完成人工复核和结构化编码，review_status均为completed。</x:v>
+        <x:v>All 20 manual reviews are complete; review_status is completed in column Z.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="16" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="B10" s="13" t="s">
-        <x:v>197</x:v>
+      <x:c r="A10" s="16" t="str">
+        <x:v>Display text</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>English claim translations come from data/claims.csv. English case titles come from assets/case-summaries-en.json. Original Chinese text remains in the source files.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="17" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="B11" s="14" t="s">
-        <x:v>199</x:v>
+      <x:c r="A11" s="17" t="str">
+        <x:v>Low risk</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>low_risk means no concern was found by the configured checks.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: restore full structured review workbook with completed status values
</commit_message>
<xml_diff>
--- a/evaluation/manual_review_20.xlsx
+++ b/evaluation/manual_review_20.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Review" sheetId="1" r:id="R8a3635ce28c14305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Notes" sheetId="2" r:id="R6b2d16431aae44a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核记录" sheetId="1" r:id="R539c21922ea6490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R5e54bd72fab342da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11,9 +11,90 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
+    <x:t xml:space="preserve">ClaimTrace manual review of the locked test set (20 records)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">All 20 records</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Case-derived</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Synthetic</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">System abstention</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">confirmed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pending</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">claim_id</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Claim text (Chinese)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Source type</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reference label</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">System output</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstained</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Top similarity</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Model reason</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement support</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Citation support</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Recommendation actionability</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Uncertainty expression</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Suggested human label</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">System assessment</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Review status</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Review note</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Citation title</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Citation URL</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM031</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">每月只花9元，这张流量卡就能不限量使用全部高速流量。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">case_derived</x:t>
   </x:si>
   <x:si>
@@ -23,127 +104,511 @@
     <x:t xml:space="preserve">high_risk</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">no</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim about unlimited high-speed data for only 9 yuan per month is similar to a previous case where a company made a false price claim regarding a mobile data card. This indicates a risk of misleading advertising.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Partial support: a low price with unlimited use is a price-and-volume promise that needs verification; a similar case can only flag the risk and cannot prove the current promise false.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partial support: the official case showed another company's 'large data volume at 9 yuan per month' did not match reality; it supports only the same-category risk and cannot prove this data card is false.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Not assessable: test_full.csv does not store the next_action field.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason uses risk wording, but the system still outputs high_risk directly and does not adequately separate analogical risk from the current facts.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Over-escalation: the reference label calls for evidence, and the system judged high risk directly.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Partial support: a low price with unlimited use is a price-and-volume promise that needs verification; a similar case can only flag the risk and cannot prove the current promise false. Citation: Partial support: the official case showed another company's 'large data volume at 9 yuan per month' did not match reality; it supports only the same-category risk and cannot prove this data card is false. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason uses risk wording, but the system still outputs high_risk directly and does not adequately separate analogical risk from the current facts. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Beijing: misleading mobile-data plan pricing</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2025/art_1212b0d62d0844d58c635269e40efe35.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM032</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">使用这套护肤品七天，就能完全消除红肿、瘙痒和痘痘。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that the skincare product can completely eliminate symptoms such as redness, itching, and acne, which is a strong treatment promise. This is similar to a case where a cosmetic was advertised as treating skin conditions, leading to consumer confusion with pharmaceuticals.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: a promise to 'completely eliminate' several skin symptoms in seven days is an explicit, absolute treatment-effect claim.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Directly relevant: the official case concerns a cosmetic advertised as treating redness, swelling, itching, stinging and acne, which closely matches the current symptoms and product type.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason explains the similar case and the medicine-confusion risk, but it does not state clearly that final publication still requires a human check against the product's facts.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Judgement consistent; citation directly relevant.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: a promise to 'completely eliminate' several skin symptoms in seven days is an explicit, absolute treatment-effect claim. Citation: Directly relevant: the official case concerns a cosmetic advertised as treating redness, swelling, itching, stinging and acne, which closely matches the current symptoms and product type. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason explains the similar case and the medicine-confusion risk, but it does not state clearly that final publication still requires a human check against the product's facts. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Hangzhou: cosmetic advertised as treating skin conditions</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM034</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">已有大量消费者亲自证明，这款果冻可以快速减肥。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests a strong cure promise for weight loss, which is a high-risk assertion without sufficient evidence to support it. Similar cases have involved unsupported health claims that were deemed illegal.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Partial support: rapid weight loss and 'consumer proof' require effectiveness evidence and proof that the testimonials are genuine; the text alone cannot establish a false claim.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Insufficient: the reason moves directly from missing evidence to high risk without explaining that the current testimonials and product effect still need verification.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Shanwei: cognitive and sleep claims for candy</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.shanwei.gov.cn/swscjdglj/zwgk/0800/dxal/content/post_1074414.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM035</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">实测证明，这款家用美容仪能够显著提升皮肤紧致度。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests a significant improvement in skin firmness, which is a strong therapeutic promise that is likely to be considered a medical claim. This type of claim is often scrutinized and can be classified as a high risk due to potential consumer deception.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Partial support: a claimed significant improvement in firmness is a verifiable efficacy claim that should have test or trial support; the input alone does not justify a high-risk finding.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Weakly relevant: the source case is about a false whitening claim for an ordinary hand wash; it shows cosmetics efficacy must have a genuine basis, but it is neither the same product nor the same effect as the firmness claim.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Insufficient: the reason summarises the firmness claim as a therapeutic promise without explaining the product category and the evidence gap.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Over-escalated with a weak citation.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Partial support: a claimed significant improvement in firmness is a verifiable efficacy claim that should have test or trial support; the input alone does not justify a high-risk finding. Citation: Weakly relevant: the source case is about a false whitening claim for an ordinary hand wash; it shows cosmetics efficacy must have a genuine basis, but it is neither the same product nor the same effect as the firmness claim. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Insufficient: the reason summarises the firmness claim as a therapeutic promise without explaining the product category and the evidence gap. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Fangxian: unsupported whitening claim for hand wash</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/ggjgs/sjdt/gzdt/art/2024/art_93bcd60c81fb4145b6698014ba162cbb.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM036</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款普通膏体可以修复身体损伤并缓解相关疾病症状。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that the ordinary ointment can repair bodily injuries and alleviate disease symptoms, which is a medical claim for a non-medical product. This aligns with previous enforcement cases where similar claims were made for ordinary products, leading to legal action.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: an ordinary ointment claiming to repair bodily injury and relieve disease symptoms is a clear expression of disease-treatment function.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Directly relevant: the official case concerns an ordinary ointment claiming disease treatment and restored mobility, which closely matches the current therapeutic promise for an ordinary ointment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason explains the risk of medical wording for ordinary products, but it should keep the boundary that a human makes the final confirmation.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: an ordinary ointment claiming to repair bodily injury and relieve disease symptoms is a clear expression of disease-treatment function. Citation: Directly relevant: the official case concerns an ordinary ointment claiming disease treatment and restored mobility, which closely matches the current therapeutic promise for an ordinary ointment. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason explains the risk of medical wording for ordinary products, but it should keep the boundary that a human makes the final confirmation. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Qingdao: treatment claims for an ordinary ointment</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2025/art_aa3fc21f7586462593b51175ba385186.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM037</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款产品可以全面改善身体机能，效果远超同类商品。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests comprehensive improvement of bodily functions, which is a strong health claim that is unsupported by evidence. Similar cases have been found where products made similar claims without scientific backing, leading to enforcement actions.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Partial support: claims of comprehensively improving bodily functions and outperforming comparable products require evidence; the current input is not enough to judge high risk directly.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly relevant: the source is a case of false health or improvement claims for ordinary food; it supports an evidence-needed judgement but is not the same as the generalised 'comprehensively improves bodily functions' claim.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Insufficient: the reason cites the lack of scientific basis but does not say that product and comparison evidence should be requested first.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Over-escalation: evidence needed is the more suitable label.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Partial support: claims of comprehensively improving bodily functions and outperforming comparable products require evidence; the current input is not enough to judge high risk directly. Citation: Partly relevant: the source is a case of false health or improvement claims for ordinary food; it supports an evidence-needed judgement but is not the same as the generalised 'comprehensively improves bodily functions' claim. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Insufficient: the reason cites the lack of scientific basis but does not say that product and comparison evidence should be requested first. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM039</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">本店销售的珍珠全部为天然珍珠，并附有真实权威证书。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim states that all pearls sold are natural and come with authentic certification. However, there is evidence of a case where fake pearls were sold as real, along with forged certification. This raises significant concerns about the authenticity of the pearls being sold.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Partial support: natural pearls and authoritative certification are product-authenticity promises that require verification of the shop's own appraisal and certificates.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Highly relevant but not direct proof: the official case does involve imitation pearls sold as genuine with forged certificates; it can only prompt verification and cannot prove this shop also falsifies.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Insufficient: the reason projects the old case onto the current product's authenticity concern without emphasising enough that it cannot directly prove anything across sellers.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Over-escalation: analogical risk is not the current fact.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Partial support: natural pearls and authoritative certification are product-authenticity promises that require verification of the shop's own appraisal and certificates. Citation: Highly relevant but not direct proof: the official case does involve imitation pearls sold as genuine with forged certificates; it can only prompt verification and cannot prove this shop also falsifies. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Insufficient: the reason projects the old case onto the current product's authenticity concern without emphasising enough that it cannot directly prove anything across sellers. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Zhuji: imitation pearls sold as genuine</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM040</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">直播间里的和田玉全部来自主播展示的矿区，来源绝对可靠。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">insufficient_evidence</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">yes</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The retrieved evidence is below the provisional similarity threshold.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Abstention supported: the mining-area origin and 'absolutely reliable' claim require supply-chain and origin documentation; abstention at a low retrieval score is reasonable.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the similarity 0.2928 is below the provisional 0.30 threshold, the system provided no source, so citation authenticity cannot be checked.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system states explicitly that it abstains because the score is below the provisional threshold; but it does not say which origin and supply-chain materials a human should verify.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstention reasonable</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Abstention supported: the mining-area origin and 'absolutely reliable' claim require supply-chain and origin documentation; abstention at a low retrieval score is reasonable. Citation: No citation: the similarity 0.2928 is below the provisional 0.30 threshold, the system provided no source, so citation authenticity cannot be checked. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system states explicitly that it abstains because the score is below the provisional threshold; but it does not say which origin and supply-chain materials a human should verify. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM042</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">权威研究和真实用户反馈证明，蜂王浆具有抗肿瘤等药理作用。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that royal jelly has anti-tumor properties, which is a medical claim that is prohibited for ordinary products. Similar cases have shown that such claims can lead to enforcement actions due to their misleading nature.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: an ordinary bee product claiming anti-tumour pharmacological effects is a clear expression of disease-treatment or medicinal efficacy.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Directly relevant: the official case states that the royal jelly 'pharmacological effects', user feedback and research-institution claims were untrue or unlawful, matching the input closely.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason notes the risk of medical claims for ordinary products, but a human still needs to check the specific product attributes and promotional context.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: an ordinary bee product claiming anti-tumour pharmacological effects is a clear expression of disease-treatment or medicinal efficacy. Citation: Directly relevant: the official case states that the royal jelly 'pharmacological effects', user feedback and research-institution claims were untrue or unlawful, matching the input closely. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason notes the risk of medical claims for ordinary products, but a human still needs to check the specific product attributes and promotional context. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Qiandaohu Chunxin: false royal-jelly claims</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2024/art_a68c3d6b97c24ec89fbb52182b9a24b8.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM044</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">每天饮用这款骆驼奶粉，就能有效控制血糖和三高问题。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that the product can control blood sugar and manage health issues related to 'three highs', which is a disease prevention or treatment claim. This is similar to a previous enforcement case where camel milk was advertised with similar health benefits, leading to legal action for making unapproved health claims.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: an ordinary food claiming to control blood sugar and the 'three highs' is an expression of disease-prevention or treatment function.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Directly relevant: the official case explicitly concerns camel-milk powder claims of 'lowering blood sugar' and 'managing the three highs', almost the same category as the input.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason explains the disease-treatment risk, but the final publication decision still requires human confirmation of product attributes and full context.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: an ordinary food claiming to control blood sugar and the 'three highs' is an expression of disease-prevention or treatment function. Citation: Directly relevant: the official case explicitly concerns camel-milk powder claims of 'lowering blood sugar' and 'managing the three highs', almost the same category as the input. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason explains the disease-treatment risk, but the final publication decision still requires human confirmation of product attributes and full context. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Yunnan Xinghao: disease claims for camel milk powder</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM076</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款笔记本可选横线页或空白页。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">synthetic</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">low_risk</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; the low-risk judgement is based only on the input text and is not legal approval.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system states it is below the threshold and abstains, but it does not distinguish an ordinary product-specification statement.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM077</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款蓝牙音箱全年累计销量突破100万台。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstention supported: annual sales above one million units is a verifiable fact that requires platform, order or sales records.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; sales authenticity must be verified separately.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system does not force a judgement on insufficient evidence, but it does not say which sales records are needed.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Abstention supported: annual sales above one million units is a verifiable fact that requires platform, order or sales records. Citation: No citation: the system abstained below the threshold and produced no source; sales authenticity must be verified separately. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system does not force a judgement on insufficient evidence, but it does not say which sales records are needed. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM078</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款普通乳饮料可以治疗贫血。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that a regular dairy drink can treat a medical condition (anemia), which is a strong cure promise and is prohibited. Similar cases have established that such claims are illegal.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: an ordinary dairy drink claiming to treat anaemia is an explicit disease-treatment promise.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly relevant: the cited case concerns ordinary food claiming to regulate blood sugar, the 'three highs' and similar disease functions; it supports the rule that ordinary food must not claim to treat disease; it is not the same case as anaemia or a dairy drink.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason explains the risk of disease-treatment claims for ordinary food, but the wording 'a similar case proves a violation' can be read as a definite conclusion about the current product.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Judgement consistent; citation supports the category-level point.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: an ordinary dairy drink claiming to treat anaemia is an explicit disease-treatment promise. Citation: Partly relevant: the cited case concerns ordinary food claiming to regulate blood sugar, the 'three highs' and similar disease functions; it supports the rule that ordinary food must not claim to treat disease; it is not the same case as anaemia or a dairy drink. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason explains the risk of disease-treatment claims for ordinary food, but the wording 'a similar case proves a violation' can be read as a definite conclusion about the current product. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Chengmai Hengsheng Hospital: health claims for beverage powder</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">https://www.samr.gov.cn/xw/zj/art/2024/art_040ee3ac2e924c1e9735c6f47fb734d9.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CLAIM079</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款雨伞有黄色和黑色两种颜色。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim simply states the available colors of the umbrella, which does not raise any configured concerns or legal issues. This is not legal approval, but the claim appears to be straightforward and factual.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: the text only describes the umbrella's colour options and triggers no configured risk; the listing must still match the physical product.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the low-risk output has no source; the colour description can be checked directly, but low risk is not legal approval.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Quite clear: the model states that no configured risk is triggered and that this is not legal approval.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Judgement consistent; no citation is acceptable here.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: the text only describes the umbrella's colour options and triggers no configured risk; the listing must still match the physical product. Citation: No citation: the low-risk output has no source; the colour description can be checked directly, but low risk is not legal approval. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Quite clear: the model states that no configured risk is triggered and that this is not legal approval. Human conclusion: the current evidence better supports low_risk.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM080</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这件防晒衣的防紫外线系数达到UPF50+。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstention supported: UPF50+ is a verifiable performance indicator that requires a test report, the applicable standard and its conditions.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; performance authenticity needs test materials.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system states it is below the threshold and abstains, but it does not point to the test standard and conditions to verify.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Abstention supported: UPF50+ is a verifiable performance indicator that requires a test report, the applicable standard and its conditions. Citation: No citation: the system abstained below the threshold and produced no source; performance authenticity needs test materials. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system states it is below the threshold and abstains, but it does not point to the test standard and conditions to verify. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM081</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款普通口香糖能够治愈牙周炎。</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">The claim suggests that a common chewing gum can cure periodontal disease, which is a strong health claim that is unsupported by evidence. Similar cases have shown that such health-related claims are considered illegal and misleading.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Supported: an ordinary chewing gum claiming to cure periodontal disease is an explicit disease-treatment promise.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly relevant: the source case concerns false health claims for ordinary food and supports the disease-treatment risk for ordinary food; it is not the same case as chewing gum or periodontal disease.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partly clear: the reason explains the risk of curing disease, but it should state that the citation supports only a category-level judgement.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Judgement consistent; citation gives partial support.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Supported: an ordinary chewing gum claiming to cure periodontal disease is an explicit disease-treatment promise. Citation: Partly relevant: the source case concerns false health claims for ordinary food and supports the disease-treatment risk for ordinary food; it is not the same case as chewing gum or periodontal disease. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Partly clear: the reason explains the risk of curing disease, but it should state that the citation supports only a category-level judgement. Human conclusion: the current evidence better supports high_risk.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM084</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">穿上这款普通袜子就能百分之百预防静脉曲张。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; the human conclusion comes from the disease-prevention and absolute-guarantee wording in the input.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clearly states the reason for abstention, but does not point out that the input itself contains strong disease-prevention signals.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM086</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款空气净化器能去除99.9%的室内微尘。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstention supported: removing 99.9% of indoor dust is a quantified performance promise that requires stated test conditions and a test report.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; quantified effects need product test materials.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system does not force a judgement on insufficient evidence, but it omits key conditions such as the test environment and particle range.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Abstention supported: removing 99.9% of indoor dust is a quantified performance promise that requires stated test conditions and a test report. Citation: No citation: the system abstained below the threshold and produced no source; quantified effects need product test materials. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system does not force a judgement on insufficient evidence, but it omits key conditions such as the test environment and particle range. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM089</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">这款水壶获得了国际设计奖。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Abstention supported: winning an international design award is a verifiable fact that requires the award name, organiser and proof of the award.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; the award claim must be verified with external materials.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clear: the system states the evidence is insufficient and abstains, but does not suggest how to verify the specific award.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Input and judgement: Abstention supported: winning an international design award is a verifiable fact that requires the award name, organiser and proof of the award. Citation: No citation: the system abstained below the threshold and produced no source; the award claim must be verified with external materials. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system states the evidence is insufficient and abstains, but does not suggest how to verify the specific award. Human conclusion: the current evidence better supports evidence_needed.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">CLAIM090</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">这款家用靠垫保证治愈腰椎间盘突出。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">No citation: the system abstained below the threshold and produced no source; the human conclusion comes from the cure guarantee in the input.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Clearly states the reason for abstention, but does not point out that the input itself contains a strong cure signal.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Usage notes</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Purpose</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">These 20 manual review records are kept for the course submission. This is a screening-quality check, not legal advice.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sample</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Ten case-derived and ten synthetic items from the locked test set; development item CLAIM072 is not included.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Label boundaries</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reference labels were written by the project author and are not official regulator labels; insufficient_evidence is the system's abstention output.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Citation checking</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Records with citations were checked against the corresponding government pages; 'partial support' means the citation supports only a category-level or analogical risk and cannot prove facts about the current seller.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Recommendation check</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">test_full.csv does not store next_action, so all 20 records are honestly marked not assessable; no recommendations were invented.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Current status</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Do not modify</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Do not change reference labels, system outputs, the locked test set or existing results files to improve the results.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Low-risk note</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">low_risk only means no configured risk was triggered; it is not legal approval; publication still requires human confirmation.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -193,12 +658,12 @@
     </x:font>
     <x:font>
       <x:sz val="9"/>
-      <x:name val="Arial"/>
+      <x:name val="宋体"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF222222"/>
-      <x:name val="Arial"/>
+      <x:name val="微软雅黑"/>
     </x:font>
   </x:fonts>
   <x:fills count="5">
@@ -371,7 +836,7 @@
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
-    <x:cellStyle name="Review body" xfId="0"/>
+    <x:cellStyle name="常规" xfId="0"/>
   </x:cellStyles>
   <x:dxfs count="3">
     <x:dxf>
@@ -417,23 +882,23 @@
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="No."/>
     <x:tableColumn id="2" name="claim_id"/>
-    <x:tableColumn id="3" name="Claim (English translation)"/>
-    <x:tableColumn id="4" name="Sample type"/>
+    <x:tableColumn id="3" name="Claim text (Chinese)"/>
+    <x:tableColumn id="4" name="Source type"/>
     <x:tableColumn id="5" name="Reference label"/>
     <x:tableColumn id="6" name="System output"/>
     <x:tableColumn id="7" name="Abstained"/>
     <x:tableColumn id="8" name="Top similarity"/>
     <x:tableColumn id="9" name="Model reason"/>
-    <x:tableColumn id="10" name="Input and rating support"/>
+    <x:tableColumn id="10" name="Input and judgement support"/>
     <x:tableColumn id="11" name="Citation support"/>
     <x:tableColumn id="12" name="Recommendation actionability"/>
-    <x:tableColumn id="13" name="Uncertainty wording"/>
-    <x:tableColumn id="14" name="Human label"/>
+    <x:tableColumn id="13" name="Uncertainty expression"/>
+    <x:tableColumn id="14" name="Suggested human label"/>
     <x:tableColumn id="15" name="System assessment"/>
     <x:tableColumn id="16" name="Review status"/>
-    <x:tableColumn id="17" name="Review conclusion"/>
-    <x:tableColumn id="18" name="Cited case (English summary title)"/>
-    <x:tableColumn id="19" name="Source URL"/>
+    <x:tableColumn id="17" name="Review note"/>
+    <x:tableColumn id="18" name="Citation title"/>
+    <x:tableColumn id="19" name="Citation URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -665,8 +1130,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18.75">
-      <x:c r="A1" s="1" t="str">
-        <x:v>ClaimTrace: Manual review of 20 locked-test claims</x:v>
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -689,7 +1154,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>Ten case-derived and ten synthetic claims were reviewed. Coded results and source links appear below.</x:v>
+        <x:v>Ten case-derived rewrites plus ten synthetic claims. All 20 records have completed manual review and structured coding; review conclusions are not legal approval, and publication still requires human confirmation.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -732,40 +1197,40 @@
       <x:c r="S3" s="2"/>
     </x:row>
     <x:row r="4" ht="13.899999618530273">
-      <x:c r="A4" s="4" t="str">
-        <x:v>Reviewed</x:v>
+      <x:c r="A4" s="4" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="5">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>Case-derived</x:v>
+      <x:c r="C4" s="5" t="s">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D4" s="5">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="str">
-        <x:v>Synthetic</x:v>
+      <x:c r="E4" s="5" t="s">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="5">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="str">
-        <x:v>Abstentions</x:v>
+      <x:c r="G4" s="5" t="s">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H4" s="5" t="n">
         <x:f>COUNTIF(F7:F26,"insufficient_evidence")</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I4" s="5" t="str">
-        <x:v>Completed</x:v>
+      <x:c r="I4" s="5" t="s">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J4" s="5" t="n">
         <x:f>COUNTIF(Z7:Z26,"completed")</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K4" s="5" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="K4" s="5" t="s">
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L4" s="6" t="n">
         <x:f>COUNTIF(Z7:Z26,"pending")</x:f>
@@ -801,62 +1266,62 @@
       <x:c r="S5" s="2"/>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="7" t="str">
-        <x:v>No.</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="str">
-        <x:v>claim_id</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="str">
-        <x:v>Claim (English translation)</x:v>
-      </x:c>
-      <x:c r="D6" s="7" t="str">
-        <x:v>Sample type</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="str">
-        <x:v>Reference label</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="str">
-        <x:v>System output</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="str">
-        <x:v>Abstained</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="str">
-        <x:v>Top similarity</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="str">
-        <x:v>Model reason</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="str">
-        <x:v>Input and rating support</x:v>
-      </x:c>
-      <x:c r="K6" s="7" t="str">
-        <x:v>Citation support</x:v>
-      </x:c>
-      <x:c r="L6" s="7" t="str">
-        <x:v>Recommendation actionability</x:v>
-      </x:c>
-      <x:c r="M6" s="7" t="str">
-        <x:v>Uncertainty wording</x:v>
-      </x:c>
-      <x:c r="N6" s="7" t="str">
-        <x:v>Human label</x:v>
-      </x:c>
-      <x:c r="O6" s="7" t="str">
-        <x:v>System assessment</x:v>
-      </x:c>
-      <x:c r="P6" s="7" t="str">
-        <x:v>Review status</x:v>
-      </x:c>
-      <x:c r="Q6" s="7" t="str">
-        <x:v>Review conclusion</x:v>
-      </x:c>
-      <x:c r="R6" s="7" t="str">
-        <x:v>Cited case (English summary title)</x:v>
-      </x:c>
-      <x:c r="S6" s="7" t="str">
-        <x:v>Source URL</x:v>
+      <x:c r="A6" s="7" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G6" s="7" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="K6" s="7" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="L6" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="M6" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="N6" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="O6" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="P6" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="Q6" s="7" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="R6" s="7" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="S6" s="7" t="s">
+        <x:v>25</x:v>
       </x:c>
       <x:c r="T6" s="19" t="str">
         <x:v>citation_present</x:v>
@@ -885,58 +1350,58 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="str">
-        <x:v>For only RMB 9 per month, this mobile data card provides unlimited high-speed data.</x:v>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="s">
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E7" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F7" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G7" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H7" s="11">
         <x:v>0.46310000000000001</x:v>
       </x:c>
       <x:c r="I7" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J7" s="8" t="str">
-        <x:v>Partial support: a low-priced unlimited data offer needs evidence of the tariff and allowance. A similar case alone does not establish that this offer is false.</x:v>
-      </x:c>
-      <x:c r="K7" s="8" t="str">
-        <x:v>Partial support: the official case found another company's CNY 9 per month data advertisement inconsistent with its actual offer. It supports a comparable risk, not a finding about this card.</x:v>
-      </x:c>
-      <x:c r="L7" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M7" s="8" t="str">
-        <x:v>Partly clear: the reason uses risk language, but the high_risk label blurs analogy with facts about this seller.</x:v>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J7" s="8" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="K7" s="8" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="L7" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M7" s="8" t="s">
+        <x:v>36</x:v>
       </x:c>
       <x:c r="N7" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O7" s="10" t="str">
-        <x:v>Overclassified: the reference label calls for evidence, while the system assigns high risk.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="s">
+        <x:v>37</x:v>
       </x:c>
       <x:c r="P7" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q7" s="8" t="str">
-        <x:v>Human review favors evidence_needed until the current price and data terms are verified.</x:v>
-      </x:c>
-      <x:c r="R7" s="8" t="str">
-        <x:v>Beijing: misleading mobile-data plan pricing</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q7" s="8" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="R7" s="8" t="s">
+        <x:v>39</x:v>
       </x:c>
       <x:c r="S7" s="8" t="s">
-        <x:v>5</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T7" s="21" t="str">
         <x:v>yes</x:v>
@@ -965,58 +1430,58 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B8" s="9" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="str">
-        <x:v>Using this skincare set for seven days will completely eliminate redness, itching and acne.</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="s">
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E8" s="9" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F8" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G8" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H8" s="11">
         <x:v>0.41060000000000002</x:v>
       </x:c>
       <x:c r="I8" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="J8" s="8" t="str">
-        <x:v>Supported: a promise to completely eliminate several skin symptoms within seven days is an explicit, absolute treatment-effect claim.</x:v>
-      </x:c>
-      <x:c r="K8" s="8" t="str">
-        <x:v>Directly relevant: the official case concerns a cosmetic advertised as treating redness, itching, stinging and acne. The product type and symptoms closely match.</x:v>
-      </x:c>
-      <x:c r="L8" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M8" s="8" t="str">
-        <x:v>Partly clear: the reason explains the similar case and medicine-confusion risk, but does not explicitly call for checking this product's facts before publication.</x:v>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="J8" s="8" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="K8" s="8" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="L8" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M8" s="8" t="s">
+        <x:v>46</x:v>
       </x:c>
       <x:c r="N8" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O8" s="10" t="str">
-        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="s">
+        <x:v>47</x:v>
       </x:c>
       <x:c r="P8" s="18" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q8" s="8" t="str">
-        <x:v>Human review agrees with high_risk because the claim guarantees treatment of skin symptoms.</x:v>
-      </x:c>
-      <x:c r="R8" s="8" t="str">
-        <x:v>Hangzhou: cosmetic advertised as treating skin conditions</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q8" s="8" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="R8" s="8" t="s">
+        <x:v>49</x:v>
       </x:c>
       <x:c r="S8" s="8" t="s">
-        <x:v>5</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T8" s="21" t="str">
         <x:v>yes</x:v>
@@ -1045,58 +1510,58 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="9" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C9" s="8" t="str">
-        <x:v>A large number of consumers have personally confirmed that this jelly produces rapid weight loss.</x:v>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="s">
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D9" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E9" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F9" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H9" s="11">
         <x:v>0.48559999999999998</x:v>
       </x:c>
       <x:c r="I9" s="8" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="J9" s="8" t="str">
-        <x:v>Partial support: rapid weight loss and claimed consumer confirmation need efficacy evidence and authentic reviews. The wording alone does not establish falsity.</x:v>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="J9" s="8" t="s">
+        <x:v>53</x:v>
       </x:c>
       <x:c r="K9" s="8" t="str">
-        <x:v>Weak match: the linked Shanwei case concerns efficacy claims for ordinary food, not jelly weight loss or fabricated user comments. It offers category-level context only.</x:v>
-      </x:c>
-      <x:c r="L9" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M9" s="8" t="str">
-        <x:v>Insufficient: the reason treats missing evidence as high risk without explaining that the current reviews and product effects still need verification.</x:v>
+        <x:v>Weakly relevant and the citation does not fully match the reason: the current link points to the Shanwei ordinary-food efficacy case, whose page contains no jelly weight-loss or fake user-review content; it can only provide category-level support for ordinary-food efficacy claims.</x:v>
+      </x:c>
+      <x:c r="L9" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M9" s="8" t="s">
+        <x:v>54</x:v>
       </x:c>
       <x:c r="N9" s="10" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="O9" s="10" t="str">
-        <x:v>Overclassified: the citation does not fully support the model's stated reason.</x:v>
+        <x:v>Over-escalated, and the current citation does not fully match the model's reason</x:v>
       </x:c>
       <x:c r="P9" s="10" t="str">
-        <x:v>Completed</x:v>
+        <x:v>completed</x:v>
       </x:c>
       <x:c r="Q9" s="8" t="str">
-        <x:v>Human review favors evidence_needed; the cited case does not establish this product's results or review authenticity.</x:v>
-      </x:c>
-      <x:c r="R9" s="8" t="str">
-        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
+        <x:v>Input and judgement: Partial support: rapid weight loss and 'consumer proof' require effectiveness evidence and proof that the testimonials are genuine; the text alone cannot establish a false claim. Citation: Weakly relevant and the citation does not fully match the reason: the current link points to the Shanwei ordinary-food efficacy case, whose page contains no jelly weight-loss or fake user-review content; it can only provide category-level support for ordinary-food efficacy claims. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Insufficient: the reason moves directly from missing evidence to high risk without explaining that the current testimonials and product effect still need verification. Human conclusion: the current evidence better supports evidence_needed.</x:v>
+      </x:c>
+      <x:c r="R9" s="8" t="s">
+        <x:v>55</x:v>
       </x:c>
       <x:c r="S9" s="8" t="s">
-        <x:v>10</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="T9" s="21" t="str">
         <x:v>yes</x:v>
@@ -1125,58 +1590,58 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B10" s="9" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C10" s="8" t="str">
-        <x:v>Testing proves that this home beauty device can significantly improve skin firmness.</x:v>
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="s">
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D10" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E10" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F10" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G10" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H10" s="11">
         <x:v>0.45450000000000002</x:v>
       </x:c>
       <x:c r="I10" s="8" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="J10" s="8" t="str">
-        <x:v>Partial support: improved skin firmness is a testable efficacy claim needing test evidence. The submitted wording alone does not establish high risk.</x:v>
-      </x:c>
-      <x:c r="K10" s="8" t="str">
-        <x:v>Weak match: the source concerns false whitening claims for ordinary hand soap, not a beauty device or skin-firmness performance.</x:v>
-      </x:c>
-      <x:c r="L10" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M10" s="8" t="str">
-        <x:v>Insufficient: the reason frames firmness as a treatment promise without addressing product type or the missing performance evidence.</x:v>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J10" s="8" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K10" s="8" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="L10" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M10" s="8" t="s">
+        <x:v>62</x:v>
       </x:c>
       <x:c r="N10" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O10" s="10" t="str">
-        <x:v>Overclassified, with a weak citation.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="s">
+        <x:v>63</x:v>
       </x:c>
       <x:c r="P10" s="18" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q10" s="8" t="str">
-        <x:v>Human review favors evidence_needed until the claimed test and performance evidence are checked.</x:v>
-      </x:c>
-      <x:c r="R10" s="8" t="str">
-        <x:v>Fangxian: unsupported whitening claim for hand wash</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q10" s="8" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="R10" s="8" t="s">
+        <x:v>65</x:v>
       </x:c>
       <x:c r="S10" s="8" t="s">
-        <x:v>13</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="T10" s="21" t="str">
         <x:v>yes</x:v>
@@ -1205,58 +1670,58 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B11" s="9" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C11" s="8" t="str">
-        <x:v>This ordinary paste can repair physical damage and relieve disease-related symptoms.</x:v>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="s">
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D11" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E11" s="9" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F11" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H11" s="11">
         <x:v>0.31209999999999999</x:v>
       </x:c>
       <x:c r="I11" s="8" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="J11" s="8" t="str">
-        <x:v>Supported: an ordinary paste claiming to repair physical damage and relieve disease symptoms makes an explicit treatment-effect claim.</x:v>
-      </x:c>
-      <x:c r="K11" s="8" t="str">
-        <x:v>Directly relevant: the official case concerns an ordinary paste promoted through disease-treatment and restored-mobility claims.</x:v>
-      </x:c>
-      <x:c r="L11" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M11" s="8" t="str">
-        <x:v>Partly clear: the reason explains the medical wording risk, but the final publication decision still requires checking the product facts.</x:v>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="J11" s="8" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="K11" s="8" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L11" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M11" s="8" t="s">
+        <x:v>72</x:v>
       </x:c>
       <x:c r="N11" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O11" s="10" t="str">
-        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O11" s="10" t="s">
+        <x:v>47</x:v>
       </x:c>
       <x:c r="P11" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q11" s="8" t="str">
-        <x:v>Human review agrees with high_risk because an ordinary paste is presented as treating disease symptoms.</x:v>
-      </x:c>
-      <x:c r="R11" s="8" t="str">
-        <x:v>Qingdao: treatment claims for an ordinary ointment</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q11" s="8" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="R11" s="8" t="s">
+        <x:v>74</x:v>
       </x:c>
       <x:c r="S11" s="8" t="s">
-        <x:v>16</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="T11" s="21" t="str">
         <x:v>yes</x:v>
@@ -1285,58 +1750,58 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B12" s="9" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C12" s="8" t="str">
-        <x:v>This product can comprehensively improve bodily functions and performs far better than comparable products.</x:v>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="s">
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D12" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E12" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F12" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G12" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H12" s="11">
         <x:v>0.36980000000000002</x:v>
       </x:c>
       <x:c r="I12" s="8" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="J12" s="8" t="str">
-        <x:v>Partial support: broad claims of improved bodily function and superiority to comparable products need evidence. The input alone does not establish high risk.</x:v>
-      </x:c>
-      <x:c r="K12" s="8" t="str">
-        <x:v>Partly relevant: the source concerns false health or improvement claims for ordinary food, but not the same broad bodily-function claim.</x:v>
-      </x:c>
-      <x:c r="L12" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M12" s="8" t="str">
-        <x:v>Insufficient: the reason cites a lack of scientific support without first calling for product and comparison evidence.</x:v>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="J12" s="8" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="K12" s="8" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L12" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M12" s="8" t="s">
+        <x:v>81</x:v>
       </x:c>
       <x:c r="N12" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O12" s="10" t="str">
-        <x:v>Overclassified: requesting supporting evidence fits the reference label better.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O12" s="10" t="s">
+        <x:v>82</x:v>
       </x:c>
       <x:c r="P12" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q12" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the performance and comparative claims.</x:v>
-      </x:c>
-      <x:c r="R12" s="8" t="str">
-        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q12" s="8" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="R12" s="8" t="s">
+        <x:v>55</x:v>
       </x:c>
       <x:c r="S12" s="8" t="s">
-        <x:v>10</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="T12" s="21" t="str">
         <x:v>yes</x:v>
@@ -1365,58 +1830,58 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B13" s="9" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C13" s="8" t="str">
-        <x:v>All pearls sold by this store are natural and are supplied with genuine authoritative certificates.</x:v>
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="s">
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D13" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E13" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F13" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G13" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H13" s="11">
         <x:v>0.73229999999999995</x:v>
       </x:c>
       <x:c r="I13" s="8" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="J13" s="8" t="str">
-        <x:v>Partial support: natural pearls and authoritative certificates are authenticity claims requiring this store's appraisal and certificate records.</x:v>
-      </x:c>
-      <x:c r="K13" s="8" t="str">
-        <x:v>Highly relevant, but not direct proof: the official case involved imitation pearls and forged certificates. It supports verification, not an allegation about this store.</x:v>
-      </x:c>
-      <x:c r="L13" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M13" s="8" t="str">
-        <x:v>Insufficient: the reason moves from an earlier seller's conduct to concern about the current goods without clearly separating the two.</x:v>
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="J13" s="8" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="K13" s="8" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="L13" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M13" s="8" t="s">
+        <x:v>89</x:v>
       </x:c>
       <x:c r="N13" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O13" s="10" t="str">
-        <x:v>Overclassified: analogous risk does not establish the current facts.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="s">
+        <x:v>90</x:v>
       </x:c>
       <x:c r="P13" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q13" s="8" t="str">
-        <x:v>Human review favors evidence_needed pending appraisal and certificate checks.</x:v>
-      </x:c>
-      <x:c r="R13" s="8" t="str">
-        <x:v>Zhuji: imitation pearls sold as genuine</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q13" s="8" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="R13" s="8" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="S13" s="8" t="s">
-        <x:v>16</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="T13" s="21" t="str">
         <x:v>yes</x:v>
@@ -1445,52 +1910,52 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="9" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C14" s="8" t="str">
-        <x:v>All Hetian jade sold in the livestream comes from the mine shown by the host and has a completely reliable origin.</x:v>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="s">
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D14" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E14" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F14" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G14" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H14" s="11">
         <x:v>0.2928</x:v>
       </x:c>
       <x:c r="I14" s="8" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J14" s="8" t="str">
-        <x:v>Human review is supported: the mine-origin and completely reliable provenance claims need supply-chain and origin records; abstention fits the low retrieval score.</x:v>
-      </x:c>
-      <x:c r="K14" s="8" t="str">
-        <x:v>No citation: the 0.2928 similarity score is below the provisional 0.30 threshold, so the system returned no source.</x:v>
-      </x:c>
-      <x:c r="L14" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M14" s="8" t="str">
-        <x:v>Clear about the threshold and human review, but it does not identify the origin and supply-chain records to check.</x:v>
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="J14" s="8" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="K14" s="8" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="L14" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M14" s="8" t="s">
+        <x:v>100</x:v>
       </x:c>
       <x:c r="N14" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O14" s="10" t="str">
-        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O14" s="10" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="P14" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q14" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the jade-origin claim.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q14" s="8" t="s">
+        <x:v>102</x:v>
       </x:c>
       <x:c r="R14" s="8"/>
       <x:c r="S14" s="8"/>
@@ -1521,58 +1986,58 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B15" s="9" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="str">
-        <x:v>Authoritative research and genuine user feedback prove that royal jelly has pharmacological effects including anti-tumour activity.</x:v>
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="s">
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D15" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E15" s="9" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F15" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G15" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H15" s="11">
         <x:v>0.43120000000000003</x:v>
       </x:c>
       <x:c r="I15" s="8" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="J15" s="8" t="str">
-        <x:v>Supported: attributing anti-tumour pharmacological effects to an ordinary bee product is an explicit disease-treatment or drug-effect claim.</x:v>
-      </x:c>
-      <x:c r="K15" s="8" t="str">
-        <x:v>Directly relevant: the official case addresses royal jelly, pharmacological effects, user feedback and research-body claims closely matching this input.</x:v>
-      </x:c>
-      <x:c r="L15" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M15" s="8" t="str">
-        <x:v>Partly clear: the reason identifies the medical claim, while the precise product and advertising context still need checking.</x:v>
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="J15" s="8" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="K15" s="8" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="L15" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M15" s="8" t="s">
+        <x:v>108</x:v>
       </x:c>
       <x:c r="N15" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O15" s="10" t="str">
-        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O15" s="10" t="s">
+        <x:v>47</x:v>
       </x:c>
       <x:c r="P15" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q15" s="8" t="str">
-        <x:v>Human review agrees with high_risk because ordinary royal jelly is presented as having pharmacological effects.</x:v>
-      </x:c>
-      <x:c r="R15" s="8" t="str">
-        <x:v>Qiandaohu Chunxin: false royal-jelly claims</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q15" s="8" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="R15" s="8" t="s">
+        <x:v>110</x:v>
       </x:c>
       <x:c r="S15" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="T15" s="21" t="str">
         <x:v>yes</x:v>
@@ -1601,58 +2066,58 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B16" s="9" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="str">
-        <x:v>Drinking this camel milk powder every day can effectively control blood sugar and other related chronic health conditions.</x:v>
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="s">
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D16" s="9" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E16" s="9" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F16" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G16" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H16" s="11">
         <x:v>0.68120000000000003</x:v>
       </x:c>
       <x:c r="I16" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="J16" s="8" t="str">
-        <x:v>Supported: ordinary food advertised as controlling blood sugar and related chronic conditions makes a disease-prevention or treatment claim.</x:v>
-      </x:c>
-      <x:c r="K16" s="8" t="str">
-        <x:v>Directly relevant: the official case involves camel milk powder advertised as lowering blood sugar and addressing the same conditions.</x:v>
-      </x:c>
-      <x:c r="L16" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M16" s="8" t="str">
-        <x:v>Partly clear: the reason identifies the disease claim, while final review still needs the product type and complete advertising context.</x:v>
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="J16" s="8" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="K16" s="8" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="L16" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M16" s="8" t="s">
+        <x:v>117</x:v>
       </x:c>
       <x:c r="N16" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O16" s="10" t="str">
-        <x:v>The system label matches the human label, and the citation is directly relevant.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O16" s="10" t="s">
+        <x:v>47</x:v>
       </x:c>
       <x:c r="P16" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q16" s="8" t="str">
-        <x:v>Human review agrees with high_risk because the milk powder is promoted for chronic conditions.</x:v>
-      </x:c>
-      <x:c r="R16" s="8" t="str">
-        <x:v>Yunnan Xinghao: disease claims for camel milk powder</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q16" s="8" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="R16" s="8" t="s">
+        <x:v>119</x:v>
       </x:c>
       <x:c r="S16" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="T16" s="21" t="str">
         <x:v>yes</x:v>
@@ -1681,52 +2146,52 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="9" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="str">
-        <x:v>This notebook is available with lined or blank pages.</x:v>
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="s">
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D17" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E17" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F17" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H17" s="11">
         <x:v>0.11409999999999999</x:v>
       </x:c>
       <x:c r="I17" s="8" t="s">
-        <x:v>23</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str">
-        <x:v>Low risk under the configured checks: this describes notebook page options. Threshold-based abstention nevertheless reduces coverage of ordinary product descriptions.</x:v>
-      </x:c>
-      <x:c r="K17" s="8" t="str">
-        <x:v>No citation: the system abstained below the threshold. The input itself supports the limited low-risk reference label.</x:v>
-      </x:c>
-      <x:c r="L17" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M17" s="8" t="str">
-        <x:v>Clear about abstention, but the system does not distinguish a routine specification from a potentially risky claim.</x:v>
+        <x:v>Low-risk supported: the text only describes notebook page specifications and involves no configured high-risk type; abstention under the current threshold follows the system rules, but it reduces coverage of low-risk samples.</x:v>
+      </x:c>
+      <x:c r="K17" s="8" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="L17" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M17" s="8" t="s">
+        <x:v>125</x:v>
       </x:c>
       <x:c r="N17" s="10" t="s">
-        <x:v>31</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="O17" s="10" t="str">
-        <x:v>Abstention follows the current threshold rule, but this low-risk item is not covered.</x:v>
+        <x:v>Abstention under the current threshold is reasonable, but the low-risk sample was not covered by the system</x:v>
       </x:c>
       <x:c r="P17" s="10" t="str">
-        <x:v>Completed</x:v>
+        <x:v>completed</x:v>
       </x:c>
       <x:c r="Q17" s="8" t="str">
-        <x:v>Human review favors low_risk for the page-format description.</x:v>
+        <x:v>Input and judgement: Low-risk supported: the text only describes notebook page specifications and involves no configured high-risk type; abstention under the current threshold follows the system rules, but it reduces coverage of low-risk samples. Citation: No citation: the system abstained below the threshold and produced no source; the low-risk judgement is based only on the input text and is not legal approval. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clear: the system states it is below the threshold and abstains, but it does not distinguish an ordinary product-specification statement. Human conclusion: the current evidence better supports low_risk.</x:v>
       </x:c>
       <x:c r="R17" s="8"/>
       <x:c r="S17" s="8"/>
@@ -1757,52 +2222,52 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B18" s="9" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="str">
-        <x:v>This Bluetooth speaker sold more than one million units in one year.</x:v>
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="s">
+        <x:v>127</x:v>
       </x:c>
       <x:c r="D18" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E18" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F18" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G18" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H18" s="11">
         <x:v>0.2661</x:v>
       </x:c>
       <x:c r="I18" s="8" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J18" s="8" t="str">
-        <x:v>Human review is supported: more than one million annual sales is a verifiable claim needing platform, order or sales records.</x:v>
-      </x:c>
-      <x:c r="K18" s="8" t="str">
-        <x:v>No citation: the system abstained below the threshold; the sales count needs independent records.</x:v>
-      </x:c>
-      <x:c r="L18" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M18" s="8" t="str">
-        <x:v>Clear about insufficient retrieval evidence, but it does not identify which sales records to check.</x:v>
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="J18" s="8" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="K18" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="L18" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M18" s="8" t="s">
+        <x:v>130</x:v>
       </x:c>
       <x:c r="N18" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O18" s="10" t="str">
-        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O18" s="10" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="P18" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q18" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the annual sales figure.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q18" s="8" t="s">
+        <x:v>131</x:v>
       </x:c>
       <x:c r="R18" s="8"/>
       <x:c r="S18" s="8"/>
@@ -1833,58 +2298,58 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B19" s="9" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="str">
-        <x:v>This ordinary milk drink can treat anaemia.</x:v>
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="s">
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D19" s="9" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="F19" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G19" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H19" s="11">
         <x:v>0.49709999999999999</x:v>
       </x:c>
       <x:c r="I19" s="8" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="J19" s="8" t="str">
-        <x:v>Supported: an ordinary milk drink advertised as treating anaemia makes an explicit disease-treatment claim.</x:v>
-      </x:c>
-      <x:c r="K19" s="8" t="str">
-        <x:v>Partly relevant: the cited case concerns disease-related claims for ordinary food, but not anaemia or this milk drink.</x:v>
-      </x:c>
-      <x:c r="L19" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M19" s="8" t="str">
-        <x:v>Partly clear: the reason identifies the treatment risk, but wording that a similar case proves wrongdoing could imply a conclusion about this product.</x:v>
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="J19" s="8" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="K19" s="8" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="L19" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M19" s="8" t="s">
+        <x:v>137</x:v>
       </x:c>
       <x:c r="N19" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O19" s="10" t="str">
-        <x:v>The system label matches the human label; the citation supports the category-level risk.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="s">
+        <x:v>138</x:v>
       </x:c>
       <x:c r="P19" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q19" s="8" t="str">
-        <x:v>Human review agrees with high_risk for the anaemia-treatment wording.</x:v>
-      </x:c>
-      <x:c r="R19" s="8" t="str">
-        <x:v>Chengmai Hengsheng Hospital: health claims for beverage powder</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q19" s="8" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="R19" s="8" t="s">
+        <x:v>140</x:v>
       </x:c>
       <x:c r="S19" s="8" t="s">
-        <x:v>35</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="T19" s="21" t="str">
         <x:v>yes</x:v>
@@ -1913,52 +2378,52 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B20" s="9" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="C20" s="8" t="str">
-        <x:v>This umbrella is available in yellow and black.</x:v>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="s">
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D20" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E20" s="9" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="F20" s="9" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="G20" s="9" t="str">
-        <x:v>No</x:v>
       </x:c>
       <x:c r="H20" s="11">
         <x:v>0.34699999999999998</x:v>
       </x:c>
       <x:c r="I20" s="8" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="J20" s="8" t="str">
-        <x:v>Supported: the claim only lists umbrella colour options and triggers no configured risk; the listing should still match the goods.</x:v>
-      </x:c>
-      <x:c r="K20" s="8" t="str">
-        <x:v>No citation: the colour description can be checked against the goods, and this low-risk result does not require a case citation.</x:v>
-      </x:c>
-      <x:c r="L20" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M20" s="8" t="str">
-        <x:v>Mostly clear: the model states that no configured risk was found and does not present the result as approval.</x:v>
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="J20" s="8" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="K20" s="8" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="L20" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M20" s="8" t="s">
+        <x:v>147</x:v>
       </x:c>
       <x:c r="N20" s="10" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="O20" s="10" t="str">
-        <x:v>The system label matches the human label; no citation is acceptable here.</x:v>
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="O20" s="10" t="s">
+        <x:v>148</x:v>
       </x:c>
       <x:c r="P20" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q20" s="8" t="str">
-        <x:v>Human review agrees with low_risk for the colour-options description.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q20" s="8" t="s">
+        <x:v>149</x:v>
       </x:c>
       <x:c r="R20" s="8"/>
       <x:c r="S20" s="8"/>
@@ -1989,52 +2454,52 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B21" s="9" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C21" s="8" t="str">
-        <x:v>This sun-protective jacket has a UPF rating of 50+.</x:v>
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="s">
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D21" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E21" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F21" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H21" s="11">
         <x:v>0.26019999999999999</x:v>
       </x:c>
       <x:c r="I21" s="8" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J21" s="8" t="str">
-        <x:v>Human review is supported: UPF 50+ is a testable performance rating needing a test report, standard and applicable conditions.</x:v>
-      </x:c>
-      <x:c r="K21" s="8" t="str">
-        <x:v>No citation: the system abstained below the threshold; the rating needs product testing records.</x:v>
-      </x:c>
-      <x:c r="L21" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M21" s="8" t="str">
-        <x:v>Clear about abstention, but it does not identify the test standard or conditions to verify.</x:v>
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="J21" s="8" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="K21" s="8" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="L21" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M21" s="8" t="s">
+        <x:v>154</x:v>
       </x:c>
       <x:c r="N21" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O21" s="10" t="str">
-        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="P21" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q21" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the UPF rating.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q21" s="8" t="s">
+        <x:v>155</x:v>
       </x:c>
       <x:c r="R21" s="8"/>
       <x:c r="S21" s="8"/>
@@ -2065,58 +2530,58 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B22" s="9" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="C22" s="8" t="str">
-        <x:v>This ordinary chewing gum can cure periodontitis.</x:v>
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="s">
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D22" s="9" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E22" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="F22" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G22" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H22" s="11">
         <x:v>0.42049999999999998</x:v>
       </x:c>
       <x:c r="I22" s="8" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J22" s="8" t="str">
-        <x:v>Supported: ordinary chewing gum claiming to cure periodontitis makes an explicit disease-treatment promise.</x:v>
-      </x:c>
-      <x:c r="K22" s="8" t="str">
-        <x:v>Partly relevant: the source concerns unsupported health effects for ordinary food, not chewing gum or periodontitis.</x:v>
-      </x:c>
-      <x:c r="L22" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M22" s="8" t="str">
-        <x:v>Partly clear: the reason identifies the cure claim, but should state that the citation supports only category-level context.</x:v>
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="J22" s="8" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="K22" s="8" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="L22" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M22" s="8" t="s">
+        <x:v>161</x:v>
       </x:c>
       <x:c r="N22" s="10" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="O22" s="10" t="str">
-        <x:v>The system label matches the human label; the citation provides partial support.</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O22" s="10" t="s">
+        <x:v>162</x:v>
       </x:c>
       <x:c r="P22" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q22" s="8" t="str">
-        <x:v>Human review agrees with high_risk because the gum is advertised as curing a disease.</x:v>
-      </x:c>
-      <x:c r="R22" s="8" t="str">
-        <x:v>Shanwei: cognitive and sleep claims for candy</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q22" s="8" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="R22" s="8" t="s">
+        <x:v>55</x:v>
       </x:c>
       <x:c r="S22" s="8" t="s">
-        <x:v>10</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="T22" s="21" t="str">
         <x:v>yes</x:v>
@@ -2145,52 +2610,52 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="9" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="C23" s="8" t="str">
-        <x:v>Wearing these ordinary socks will prevent varicose veins with 100% certainty.</x:v>
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="s">
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D23" s="9" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E23" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="F23" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H23" s="11">
         <x:v>0.28810000000000002</x:v>
       </x:c>
       <x:c r="I23" s="8" t="s">
-        <x:v>23</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="J23" s="8" t="str">
-        <x:v>Abstention follows the threshold rule, but it misses an obvious signal: ordinary socks promising 100% prevention of varicose veins make an absolute disease-prevention claim.</x:v>
-      </x:c>
-      <x:c r="K23" s="8" t="str">
-        <x:v>No citation: retrieval was below the threshold. The human label follows from the disease-prevention and absolute-guarantee wording.</x:v>
-      </x:c>
-      <x:c r="L23" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M23" s="8" t="str">
-        <x:v>Clear about why the system abstained, but it does not flag the strong prevention claim already present in the input.</x:v>
+        <x:v>Abstention follows the current threshold mechanism, but the rules did not prioritise an obvious risk: an ordinary sock that 'prevents' disease 'one hundred percent' is a strong absolute disease-prevention promise and a human should judge it high risk.</x:v>
+      </x:c>
+      <x:c r="K23" s="8" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="L23" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M23" s="8" t="s">
+        <x:v>167</x:v>
       </x:c>
       <x:c r="N23" s="10" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="O23" s="10" t="str">
-        <x:v>Abstention follows the threshold rule, but the rules miss disease prevention and an absolute guarantee.</x:v>
+        <x:v>Abstention follows the current threshold mechanism, but the rules did not prioritise the disease-prevention and absolute-guarantee wording</x:v>
       </x:c>
       <x:c r="P23" s="10" t="str">
-        <x:v>Completed</x:v>
+        <x:v>completed</x:v>
       </x:c>
       <x:c r="Q23" s="8" t="str">
-        <x:v>Human review favors high_risk for the 100% disease-prevention promise.</x:v>
+        <x:v>Input and judgement: Abstention follows the current threshold mechanism, but the rules did not prioritise an obvious risk: an ordinary sock that 'prevents' disease 'one hundred percent' is a strong absolute disease-prevention promise and a human should judge it high risk. Citation: No citation: the system abstained below the threshold and produced no source; the human conclusion comes from the disease-prevention and absolute-guarantee wording in the input. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clearly states the reason for abstention, but does not point out that the input itself contains strong disease-prevention signals. Human conclusion: the current evidence better supports high_risk.</x:v>
       </x:c>
       <x:c r="R23" s="8"/>
       <x:c r="S23" s="8"/>
@@ -2221,52 +2686,52 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B24" s="9" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="C24" s="8" t="str">
-        <x:v>This air purifier removes 99.9% of fine indoor dust.</x:v>
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="s">
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D24" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E24" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F24" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G24" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H24" s="11">
         <x:v>0.29170000000000001</x:v>
       </x:c>
       <x:c r="I24" s="8" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J24" s="8" t="str">
-        <x:v>Human review is supported: a 99.9% indoor dust-removal claim needs defined test conditions and a performance report.</x:v>
-      </x:c>
-      <x:c r="K24" s="8" t="str">
-        <x:v>No citation: the system abstained below the threshold; quantified efficacy needs product-test evidence.</x:v>
-      </x:c>
-      <x:c r="L24" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M24" s="8" t="str">
-        <x:v>Clear about abstention, but it does not identify the test environment or particle range.</x:v>
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="J24" s="8" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="K24" s="8" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="L24" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M24" s="8" t="s">
+        <x:v>172</x:v>
       </x:c>
       <x:c r="N24" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O24" s="10" t="str">
-        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O24" s="10" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="P24" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q24" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the quantified removal claim.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q24" s="8" t="s">
+        <x:v>173</x:v>
       </x:c>
       <x:c r="R24" s="8"/>
       <x:c r="S24" s="8"/>
@@ -2297,52 +2762,52 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B25" s="9" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C25" s="8" t="str">
-        <x:v>This water bottle received an international design award.</x:v>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="C25" s="8" t="s">
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D25" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E25" s="9" t="s">
-        <x:v>2</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F25" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G25" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H25" s="11">
         <x:v>0.28570000000000001</x:v>
       </x:c>
       <x:c r="I25" s="8" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J25" s="8" t="str">
-        <x:v>Human review is supported: an international design award is a verifiable fact needing the award name, organiser and winner record.</x:v>
-      </x:c>
-      <x:c r="K25" s="8" t="str">
-        <x:v>No citation: the system abstained below the threshold; award authenticity needs an external record.</x:v>
-      </x:c>
-      <x:c r="L25" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M25" s="8" t="str">
-        <x:v>Clear about abstention, but it does not point to the specific award record to check.</x:v>
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="J25" s="8" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="K25" s="8" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="L25" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M25" s="8" t="s">
+        <x:v>178</x:v>
       </x:c>
       <x:c r="N25" s="10" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O25" s="10" t="str">
-        <x:v>Abstention is consistent with the current retrieval rule.</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="P25" s="10" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="Q25" s="8" t="str">
-        <x:v>Human review favors evidence_needed for the award claim.</x:v>
+        <x:v>completed</x:v>
+      </x:c>
+      <x:c r="Q25" s="8" t="s">
+        <x:v>179</x:v>
       </x:c>
       <x:c r="R25" s="8"/>
       <x:c r="S25" s="8"/>
@@ -2373,52 +2838,52 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B26" s="9" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C26" s="8" t="str">
-        <x:v>This household cushion guarantees a cure for a herniated lumbar disc.</x:v>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="C26" s="8" t="s">
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D26" s="9" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E26" s="9" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="F26" s="9" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G26" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="s">
+        <x:v>96</x:v>
       </x:c>
       <x:c r="H26" s="11">
         <x:v>0.17299999999999999</x:v>
       </x:c>
       <x:c r="I26" s="8" t="s">
-        <x:v>23</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="J26" s="8" t="str">
-        <x:v>Abstention follows the threshold rule, but it misses an obvious signal: a household cushion promising a cure for a herniated disc makes a strong treatment claim.</x:v>
-      </x:c>
-      <x:c r="K26" s="8" t="str">
-        <x:v>No citation: retrieval was below the threshold. The human label follows from the guaranteed-cure wording in the input.</x:v>
-      </x:c>
-      <x:c r="L26" s="8" t="str">
-        <x:v>Not assessable: historical test_full.csv did not record next_action.</x:v>
-      </x:c>
-      <x:c r="M26" s="8" t="str">
-        <x:v>Clear about why the system abstained, but it does not flag the cure guarantee already present in the input.</x:v>
+        <x:v>Abstention follows the current threshold mechanism, but the rules did not prioritise an obvious risk: a household cushion that 'guarantees a cure' for disease is a strong treatment promise and a human should judge it high risk.</x:v>
+      </x:c>
+      <x:c r="K26" s="8" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="L26" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M26" s="8" t="s">
+        <x:v>183</x:v>
       </x:c>
       <x:c r="N26" s="10" t="s">
-        <x:v>3</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="O26" s="10" t="str">
-        <x:v>Abstention follows the threshold rule, but the rules miss the explicit cure guarantee.</x:v>
+        <x:v>Abstention follows the current threshold mechanism, but the rules did not prioritise the obvious cure guarantee</x:v>
       </x:c>
       <x:c r="P26" s="10" t="str">
-        <x:v>Completed</x:v>
+        <x:v>completed</x:v>
       </x:c>
       <x:c r="Q26" s="8" t="str">
-        <x:v>Human review favors high_risk for the guaranteed cure.</x:v>
+        <x:v>Input and judgement: Abstention follows the current threshold mechanism, but the rules did not prioritise an obvious risk: a household cushion that 'guarantees a cure' for disease is a strong treatment promise and a human should judge it high risk. Citation: No citation: the system abstained below the threshold and produced no source; the human conclusion comes from the cure guarantee in the input. Recommendation actionability: Not assessable: test_full.csv does not store the next_action field. Uncertainty: Clearly states the reason for abstention, but does not point out that the input itself contains a strong cure signal. Human conclusion: the current evidence better supports high_risk.</x:v>
       </x:c>
       <x:c r="R26" s="8"/>
       <x:c r="S26" s="8"/>
@@ -2446,13 +2911,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="P7:P26">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Completed"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Pending"/>
-    <x:cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Needs revision"/>
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="已确认"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="待确认"/>
+    <x:cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="needs_revision"/>
   </x:conditionalFormatting>
   <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="P7:P26">
-      <x:formula1>"Completed,Pending,Needs revision"</x:formula1>
+      <x:formula1>"pending,completed,needs_revision"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="T7:T26">
       <x:formula1>"yes,no,uncertain"</x:formula1>
@@ -2475,7 +2940,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78fa3220e44f4c5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e20956d4a224274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2492,8 +2957,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18.75">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Review notes</x:v>
+      <x:c r="A1" s="1" t="s">
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
     </x:row>
@@ -2502,75 +2967,75 @@
       <x:c r="B2" s="2"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="15" t="str">
-        <x:v>Purpose</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>Manual quality review of 20 locked-test results.</x:v>
+      <x:c r="A3" s="15" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="s">
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>Sample</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Ten case-derived and ten synthetic test claims.</x:v>
+      <x:c r="A4" s="16" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="s">
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="16" t="str">
-        <x:v>Reference labels</x:v>
-      </x:c>
-      <x:c r="B5" s="13" t="str">
-        <x:v>Project-defined labels support comparison. insufficient_evidence is an abstention, not a reference label.</x:v>
+      <x:c r="A5" s="16" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="s">
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="16" t="str">
-        <x:v>Citation checks</x:v>
-      </x:c>
-      <x:c r="B6" s="13" t="str">
-        <x:v>Present citations were checked against source pages. Partial support indicates comparable risk, not a finding about the current seller.</x:v>
+      <x:c r="A6" s="16" t="s">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="s">
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="16" t="str">
-        <x:v>Actionability</x:v>
-      </x:c>
-      <x:c r="B7" s="13" t="str">
-        <x:v>Historical test_full.csv lacks next_action; actionability is not_applicable for all 20 reviews.</x:v>
+      <x:c r="A7" s="16" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="s">
+        <x:v>194</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>Coded fields</x:v>
+        <x:v>Structured fields</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>Columns T-Z retain the structured review codes. A missing citation is coded not_applicable for citation_supported.</x:v>
+        <x:v>Columns T to Z of the review records hold the structured results. citation_supported, reason_supported and uncertainty_clear are based on completed manual review conclusions; citation_supported is marked not_applicable for records without a citation.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="16" t="str">
-        <x:v>Status</x:v>
+      <x:c r="A9" s="16" t="s">
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>All 20 manual reviews are complete; review_status is completed in column Z.</x:v>
+        <x:v>All 20 records have completed manual review and structured coding; review_status is completed for all.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="16" t="str">
-        <x:v>Display text</x:v>
-      </x:c>
-      <x:c r="B10" s="13" t="str">
-        <x:v>English claim translations come from data/claims.csv. English case titles come from assets/case-summaries-en.json. Original Chinese text remains in the source files.</x:v>
+      <x:c r="A10" s="16" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="s">
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="17" t="str">
-        <x:v>Low risk</x:v>
-      </x:c>
-      <x:c r="B11" s="14" t="str">
-        <x:v>low_risk means no concern was found by the configured checks.</x:v>
+      <x:c r="A11" s="17" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="s">
+        <x:v>199</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Use English worksheet names in review evidence
</commit_message>
<xml_diff>
--- a/evaluation/manual_review_20.xlsx
+++ b/evaluation/manual_review_20.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核记录" sheetId="1" r:id="R539c21922ea6490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R5e54bd72fab342da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Review" sheetId="1" r:id="R539c21922ea6490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usage Notes" sheetId="2" r:id="R5e54bd72fab342da"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>